<commit_message>
added data as of 48 group stage matches 24/06/26
</commit_message>
<xml_diff>
--- a/data/WorldCup2026.xlsx
+++ b/data/WorldCup2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ee16c21b72f3fde9/Documents/Football Fortunes/All data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="162" documentId="8_{9D3D8A05-EEFD-4F90-A3C5-55C1E757FCE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FE2332F-1763-4528-AF5B-0BE22688E32F}"/>
+  <xr:revisionPtr revIDLastSave="170" documentId="8_{9D3D8A05-EEFD-4F90-A3C5-55C1E757FCE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95330EEB-27A4-410B-8772-81AD9AFCF4C8}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{95D741F4-B12C-45C7-A97C-F95A56A544CF}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2832" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2928" uniqueCount="267">
   <si>
     <t>Home</t>
   </si>
@@ -850,7 +850,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -877,6 +877,12 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -926,6 +932,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1225,7 +1235,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73F33CE9-0917-4340-92ED-8B6CE132D95A}">
-  <dimension ref="A1:AP25"/>
+  <dimension ref="A1:AP49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.54296875" bestFit="1" customWidth="1"/>
@@ -4175,11 +4185,2796 @@
         <v>1.31</v>
       </c>
     </row>
+    <row r="26" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>266</v>
+      </c>
+      <c r="B26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" t="s">
+        <v>85</v>
+      </c>
+      <c r="D26" s="1">
+        <v>46191</v>
+      </c>
+      <c r="E26" s="7">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>1</v>
+      </c>
+      <c r="P26" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q26">
+        <v>14</v>
+      </c>
+      <c r="R26">
+        <v>17</v>
+      </c>
+      <c r="S26">
+        <v>3</v>
+      </c>
+      <c r="T26">
+        <v>4</v>
+      </c>
+      <c r="U26">
+        <v>12</v>
+      </c>
+      <c r="V26">
+        <v>10</v>
+      </c>
+      <c r="W26">
+        <v>5</v>
+      </c>
+      <c r="X26">
+        <v>5</v>
+      </c>
+      <c r="Y26">
+        <v>1</v>
+      </c>
+      <c r="Z26">
+        <v>2</v>
+      </c>
+      <c r="AA26">
+        <v>0</v>
+      </c>
+      <c r="AB26">
+        <v>0</v>
+      </c>
+      <c r="AC26">
+        <v>1.02</v>
+      </c>
+      <c r="AD26">
+        <v>1.38</v>
+      </c>
+      <c r="AE26">
+        <v>1.85</v>
+      </c>
+      <c r="AF26">
+        <v>3.5</v>
+      </c>
+      <c r="AG26">
+        <v>4.2</v>
+      </c>
+      <c r="AH26">
+        <v>1.97</v>
+      </c>
+      <c r="AI26">
+        <v>3.5</v>
+      </c>
+      <c r="AJ26">
+        <v>4.7</v>
+      </c>
+      <c r="AK26">
+        <v>1.88</v>
+      </c>
+      <c r="AL26">
+        <v>3.55</v>
+      </c>
+      <c r="AM26">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="AN26">
+        <v>1.84</v>
+      </c>
+      <c r="AO26">
+        <v>3.41</v>
+      </c>
+      <c r="AP26">
+        <v>4.33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>266</v>
+      </c>
+      <c r="B27" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="1">
+        <v>46191</v>
+      </c>
+      <c r="E27" s="7">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F27">
+        <v>4</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>4</v>
+      </c>
+      <c r="K27">
+        <v>1</v>
+      </c>
+      <c r="P27" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q27">
+        <v>13</v>
+      </c>
+      <c r="R27">
+        <v>5</v>
+      </c>
+      <c r="S27">
+        <v>7</v>
+      </c>
+      <c r="T27">
+        <v>3</v>
+      </c>
+      <c r="U27">
+        <v>7</v>
+      </c>
+      <c r="V27">
+        <v>18</v>
+      </c>
+      <c r="W27">
+        <v>7</v>
+      </c>
+      <c r="X27">
+        <v>3</v>
+      </c>
+      <c r="Y27">
+        <v>1</v>
+      </c>
+      <c r="Z27">
+        <v>2</v>
+      </c>
+      <c r="AA27">
+        <v>0</v>
+      </c>
+      <c r="AB27">
+        <v>1</v>
+      </c>
+      <c r="AC27">
+        <v>2.06</v>
+      </c>
+      <c r="AD27">
+        <v>0.23</v>
+      </c>
+      <c r="AE27">
+        <v>1.53</v>
+      </c>
+      <c r="AF27">
+        <v>4</v>
+      </c>
+      <c r="AG27">
+        <v>6.5</v>
+      </c>
+      <c r="AH27">
+        <v>1.58</v>
+      </c>
+      <c r="AI27">
+        <v>4.3</v>
+      </c>
+      <c r="AJ27">
+        <v>7</v>
+      </c>
+      <c r="AK27">
+        <v>1.55</v>
+      </c>
+      <c r="AL27">
+        <v>4.2</v>
+      </c>
+      <c r="AM27">
+        <v>6.5</v>
+      </c>
+      <c r="AN27">
+        <v>1.52</v>
+      </c>
+      <c r="AO27">
+        <v>4.12</v>
+      </c>
+      <c r="AP27">
+        <v>6.15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>266</v>
+      </c>
+      <c r="B28" t="s">
+        <v>258</v>
+      </c>
+      <c r="C28" t="s">
+        <v>84</v>
+      </c>
+      <c r="D28" s="1">
+        <v>46191</v>
+      </c>
+      <c r="E28" s="7">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="F28">
+        <v>6</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>3</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>3</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+      <c r="P28" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q28">
+        <v>32</v>
+      </c>
+      <c r="R28">
+        <v>2</v>
+      </c>
+      <c r="S28">
+        <v>10</v>
+      </c>
+      <c r="T28">
+        <v>0</v>
+      </c>
+      <c r="U28">
+        <v>9</v>
+      </c>
+      <c r="V28">
+        <v>10</v>
+      </c>
+      <c r="W28">
+        <v>19</v>
+      </c>
+      <c r="X28">
+        <v>1</v>
+      </c>
+      <c r="Y28">
+        <v>1</v>
+      </c>
+      <c r="Z28">
+        <v>1</v>
+      </c>
+      <c r="AA28">
+        <v>0</v>
+      </c>
+      <c r="AB28">
+        <v>2</v>
+      </c>
+      <c r="AC28">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="AD28">
+        <v>0.22</v>
+      </c>
+      <c r="AE28">
+        <v>1.25</v>
+      </c>
+      <c r="AF28">
+        <v>6</v>
+      </c>
+      <c r="AG28">
+        <v>12</v>
+      </c>
+      <c r="AH28">
+        <v>1.27</v>
+      </c>
+      <c r="AI28">
+        <v>6.4</v>
+      </c>
+      <c r="AJ28">
+        <v>15.5</v>
+      </c>
+      <c r="AK28">
+        <v>1.29</v>
+      </c>
+      <c r="AL28">
+        <v>6.5</v>
+      </c>
+      <c r="AM28">
+        <v>13.5</v>
+      </c>
+      <c r="AN28">
+        <v>1.25</v>
+      </c>
+      <c r="AO28">
+        <v>5.84</v>
+      </c>
+      <c r="AP28">
+        <v>11.38</v>
+      </c>
+    </row>
+    <row r="29" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>266</v>
+      </c>
+      <c r="B29" t="s">
+        <v>253</v>
+      </c>
+      <c r="C29" t="s">
+        <v>158</v>
+      </c>
+      <c r="D29" s="1">
+        <v>46192</v>
+      </c>
+      <c r="E29" s="7">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="F29">
+        <v>1</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>0</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="J29">
+        <v>1</v>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="P29" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q29">
+        <v>8</v>
+      </c>
+      <c r="R29">
+        <v>9</v>
+      </c>
+      <c r="S29">
+        <v>4</v>
+      </c>
+      <c r="T29">
+        <v>2</v>
+      </c>
+      <c r="U29">
+        <v>9</v>
+      </c>
+      <c r="V29">
+        <v>7</v>
+      </c>
+      <c r="W29">
+        <v>0</v>
+      </c>
+      <c r="X29">
+        <v>2</v>
+      </c>
+      <c r="Y29">
+        <v>0</v>
+      </c>
+      <c r="Z29">
+        <v>2</v>
+      </c>
+      <c r="AA29">
+        <v>0</v>
+      </c>
+      <c r="AB29">
+        <v>0</v>
+      </c>
+      <c r="AC29">
+        <v>0.52</v>
+      </c>
+      <c r="AD29">
+        <v>0.91</v>
+      </c>
+      <c r="AE29">
+        <v>2</v>
+      </c>
+      <c r="AF29">
+        <v>3.25</v>
+      </c>
+      <c r="AG29">
+        <v>4</v>
+      </c>
+      <c r="AH29">
+        <v>2.12</v>
+      </c>
+      <c r="AI29">
+        <v>3.2</v>
+      </c>
+      <c r="AJ29">
+        <v>4.5</v>
+      </c>
+      <c r="AK29">
+        <v>2.13</v>
+      </c>
+      <c r="AL29">
+        <v>3.3</v>
+      </c>
+      <c r="AM29">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AN29">
+        <v>2.02</v>
+      </c>
+      <c r="AO29">
+        <v>3.19</v>
+      </c>
+      <c r="AP29">
+        <v>3.94</v>
+      </c>
+    </row>
+    <row r="30" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>266</v>
+      </c>
+      <c r="B30" t="s">
+        <v>257</v>
+      </c>
+      <c r="C30" t="s">
+        <v>149</v>
+      </c>
+      <c r="D30" s="1">
+        <v>46192</v>
+      </c>
+      <c r="E30" s="7">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F30">
+        <v>2</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30">
+        <v>2</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+      <c r="P30" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q30">
+        <v>10</v>
+      </c>
+      <c r="R30">
+        <v>5</v>
+      </c>
+      <c r="S30">
+        <v>2</v>
+      </c>
+      <c r="T30">
+        <v>2</v>
+      </c>
+      <c r="U30">
+        <v>12</v>
+      </c>
+      <c r="V30">
+        <v>16</v>
+      </c>
+      <c r="W30">
+        <v>7</v>
+      </c>
+      <c r="X30">
+        <v>4</v>
+      </c>
+      <c r="Y30">
+        <v>3</v>
+      </c>
+      <c r="Z30">
+        <v>4</v>
+      </c>
+      <c r="AA30">
+        <v>0</v>
+      </c>
+      <c r="AB30">
+        <v>0</v>
+      </c>
+      <c r="AC30">
+        <v>1.08</v>
+      </c>
+      <c r="AD30">
+        <v>0.34</v>
+      </c>
+      <c r="AE30">
+        <v>1.53</v>
+      </c>
+      <c r="AF30">
+        <v>4.33</v>
+      </c>
+      <c r="AG30">
+        <v>5.75</v>
+      </c>
+      <c r="AH30">
+        <v>1.61</v>
+      </c>
+      <c r="AI30">
+        <v>4.5</v>
+      </c>
+      <c r="AJ30">
+        <v>6</v>
+      </c>
+      <c r="AK30">
+        <v>1.61</v>
+      </c>
+      <c r="AL30">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="AM30">
+        <v>6.5</v>
+      </c>
+      <c r="AN30">
+        <v>1.55</v>
+      </c>
+      <c r="AO30">
+        <v>4.08</v>
+      </c>
+      <c r="AP30">
+        <v>5.79</v>
+      </c>
+    </row>
+    <row r="31" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>266</v>
+      </c>
+      <c r="B31" t="s">
+        <v>40</v>
+      </c>
+      <c r="C31" t="s">
+        <v>76</v>
+      </c>
+      <c r="D31" s="1">
+        <v>46192</v>
+      </c>
+      <c r="E31" s="7">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31">
+        <v>1</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <v>1</v>
+      </c>
+      <c r="J31">
+        <v>0</v>
+      </c>
+      <c r="K31">
+        <v>0</v>
+      </c>
+      <c r="P31" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q31">
+        <v>6</v>
+      </c>
+      <c r="R31">
+        <v>12</v>
+      </c>
+      <c r="S31">
+        <v>0</v>
+      </c>
+      <c r="T31">
+        <v>2</v>
+      </c>
+      <c r="U31">
+        <v>11</v>
+      </c>
+      <c r="V31">
+        <v>8</v>
+      </c>
+      <c r="W31">
+        <v>2</v>
+      </c>
+      <c r="X31">
+        <v>5</v>
+      </c>
+      <c r="Y31">
+        <v>1</v>
+      </c>
+      <c r="Z31">
+        <v>1</v>
+      </c>
+      <c r="AA31">
+        <v>0</v>
+      </c>
+      <c r="AB31">
+        <v>0</v>
+      </c>
+      <c r="AC31">
+        <v>0.52</v>
+      </c>
+      <c r="AD31">
+        <v>1</v>
+      </c>
+      <c r="AE31">
+        <v>5.25</v>
+      </c>
+      <c r="AF31">
+        <v>3.75</v>
+      </c>
+      <c r="AG31">
+        <v>1.67</v>
+      </c>
+      <c r="AH31">
+        <v>6.2</v>
+      </c>
+      <c r="AI31">
+        <v>3.8</v>
+      </c>
+      <c r="AJ31">
+        <v>1.72</v>
+      </c>
+      <c r="AK31">
+        <v>5.8</v>
+      </c>
+      <c r="AL31">
+        <v>3.8</v>
+      </c>
+      <c r="AM31">
+        <v>1.72</v>
+      </c>
+      <c r="AN31">
+        <v>5.42</v>
+      </c>
+      <c r="AO31">
+        <v>3.61</v>
+      </c>
+      <c r="AP31">
+        <v>1.67</v>
+      </c>
+    </row>
+    <row r="32" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>266</v>
+      </c>
+      <c r="B32" t="s">
+        <v>128</v>
+      </c>
+      <c r="C32" t="s">
+        <v>31</v>
+      </c>
+      <c r="D32" s="1">
+        <v>46193</v>
+      </c>
+      <c r="E32" s="7">
+        <v>6.25E-2</v>
+      </c>
+      <c r="F32">
+        <v>3</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32">
+        <v>3</v>
+      </c>
+      <c r="I32">
+        <v>0</v>
+      </c>
+      <c r="J32">
+        <v>0</v>
+      </c>
+      <c r="K32">
+        <v>0</v>
+      </c>
+      <c r="P32" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q32">
+        <v>8</v>
+      </c>
+      <c r="R32">
+        <v>7</v>
+      </c>
+      <c r="S32">
+        <v>5</v>
+      </c>
+      <c r="T32">
+        <v>3</v>
+      </c>
+      <c r="U32">
+        <v>13</v>
+      </c>
+      <c r="V32">
+        <v>14</v>
+      </c>
+      <c r="W32">
+        <v>4</v>
+      </c>
+      <c r="X32">
+        <v>4</v>
+      </c>
+      <c r="Y32">
+        <v>1</v>
+      </c>
+      <c r="Z32">
+        <v>3</v>
+      </c>
+      <c r="AA32">
+        <v>0</v>
+      </c>
+      <c r="AB32">
+        <v>0</v>
+      </c>
+      <c r="AC32">
+        <v>1.75</v>
+      </c>
+      <c r="AD32">
+        <v>0.23</v>
+      </c>
+      <c r="AE32">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AF32">
+        <v>11</v>
+      </c>
+      <c r="AG32">
+        <v>21</v>
+      </c>
+      <c r="AH32">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="AI32">
+        <v>12.5</v>
+      </c>
+      <c r="AJ32">
+        <v>22</v>
+      </c>
+      <c r="AK32">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="AL32">
+        <v>11.5</v>
+      </c>
+      <c r="AM32">
+        <v>27</v>
+      </c>
+      <c r="AN32">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="AO32">
+        <v>10.41</v>
+      </c>
+      <c r="AP32">
+        <v>22.75</v>
+      </c>
+    </row>
+    <row r="33" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>266</v>
+      </c>
+      <c r="B33" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" t="s">
+        <v>134</v>
+      </c>
+      <c r="D33" s="1">
+        <v>46193</v>
+      </c>
+      <c r="E33" s="7">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>1</v>
+      </c>
+      <c r="H33">
+        <v>0</v>
+      </c>
+      <c r="I33">
+        <v>1</v>
+      </c>
+      <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
+        <v>0</v>
+      </c>
+      <c r="P33" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q33">
+        <v>32</v>
+      </c>
+      <c r="R33">
+        <v>7</v>
+      </c>
+      <c r="S33">
+        <v>5</v>
+      </c>
+      <c r="T33">
+        <v>2</v>
+      </c>
+      <c r="U33">
+        <v>14</v>
+      </c>
+      <c r="V33">
+        <v>15</v>
+      </c>
+      <c r="W33">
+        <v>12</v>
+      </c>
+      <c r="X33">
+        <v>0</v>
+      </c>
+      <c r="Y33">
+        <v>1</v>
+      </c>
+      <c r="Z33">
+        <v>1</v>
+      </c>
+      <c r="AA33">
+        <v>0</v>
+      </c>
+      <c r="AB33">
+        <v>1</v>
+      </c>
+      <c r="AC33">
+        <v>2.17</v>
+      </c>
+      <c r="AD33">
+        <v>0.33</v>
+      </c>
+      <c r="AE33">
+        <v>2.1</v>
+      </c>
+      <c r="AF33">
+        <v>3.3</v>
+      </c>
+      <c r="AG33">
+        <v>3.6</v>
+      </c>
+      <c r="AH33">
+        <v>2.14</v>
+      </c>
+      <c r="AI33">
+        <v>3.4</v>
+      </c>
+      <c r="AJ33">
+        <v>4</v>
+      </c>
+      <c r="AK33">
+        <v>2.1</v>
+      </c>
+      <c r="AL33">
+        <v>3.45</v>
+      </c>
+      <c r="AM33">
+        <v>4</v>
+      </c>
+      <c r="AN33">
+        <v>2.02</v>
+      </c>
+      <c r="AO33">
+        <v>3.32</v>
+      </c>
+      <c r="AP33">
+        <v>3.72</v>
+      </c>
+    </row>
+    <row r="34" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>266</v>
+      </c>
+      <c r="B34" t="s">
+        <v>50</v>
+      </c>
+      <c r="C34" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="1">
+        <v>46193</v>
+      </c>
+      <c r="E34" s="7">
+        <v>0.75</v>
+      </c>
+      <c r="F34">
+        <v>5</v>
+      </c>
+      <c r="G34">
+        <v>1</v>
+      </c>
+      <c r="H34">
+        <v>2</v>
+      </c>
+      <c r="I34">
+        <v>0</v>
+      </c>
+      <c r="J34">
+        <v>3</v>
+      </c>
+      <c r="K34">
+        <v>1</v>
+      </c>
+      <c r="P34" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q34">
+        <v>10</v>
+      </c>
+      <c r="R34">
+        <v>16</v>
+      </c>
+      <c r="S34">
+        <v>7</v>
+      </c>
+      <c r="T34">
+        <v>8</v>
+      </c>
+      <c r="U34">
+        <v>9</v>
+      </c>
+      <c r="V34">
+        <v>12</v>
+      </c>
+      <c r="W34">
+        <v>2</v>
+      </c>
+      <c r="X34">
+        <v>5</v>
+      </c>
+      <c r="Y34">
+        <v>0</v>
+      </c>
+      <c r="Z34">
+        <v>3</v>
+      </c>
+      <c r="AA34">
+        <v>0</v>
+      </c>
+      <c r="AB34">
+        <v>0</v>
+      </c>
+      <c r="AC34">
+        <v>2.6</v>
+      </c>
+      <c r="AD34">
+        <v>1.01</v>
+      </c>
+      <c r="AE34">
+        <v>1.7</v>
+      </c>
+      <c r="AF34">
+        <v>4</v>
+      </c>
+      <c r="AG34">
+        <v>4.75</v>
+      </c>
+      <c r="AH34">
+        <v>1.76</v>
+      </c>
+      <c r="AI34">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AJ34">
+        <v>5.2</v>
+      </c>
+      <c r="AK34">
+        <v>1.71</v>
+      </c>
+      <c r="AL34">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AM34">
+        <v>5</v>
+      </c>
+      <c r="AN34">
+        <v>1.68</v>
+      </c>
+      <c r="AO34">
+        <v>3.96</v>
+      </c>
+      <c r="AP34">
+        <v>4.68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>266</v>
+      </c>
+      <c r="B35" t="s">
+        <v>49</v>
+      </c>
+      <c r="C35" t="s">
+        <v>79</v>
+      </c>
+      <c r="D35" s="1">
+        <v>46193</v>
+      </c>
+      <c r="E35" s="7">
+        <v>0.875</v>
+      </c>
+      <c r="F35">
+        <v>2</v>
+      </c>
+      <c r="G35">
+        <v>1</v>
+      </c>
+      <c r="H35">
+        <v>0</v>
+      </c>
+      <c r="I35">
+        <v>1</v>
+      </c>
+      <c r="J35">
+        <v>2</v>
+      </c>
+      <c r="K35">
+        <v>0</v>
+      </c>
+      <c r="P35" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q35">
+        <v>16</v>
+      </c>
+      <c r="R35">
+        <v>9</v>
+      </c>
+      <c r="S35">
+        <v>7</v>
+      </c>
+      <c r="T35">
+        <v>2</v>
+      </c>
+      <c r="U35">
+        <v>5</v>
+      </c>
+      <c r="V35">
+        <v>7</v>
+      </c>
+      <c r="W35">
+        <v>8</v>
+      </c>
+      <c r="X35">
+        <v>3</v>
+      </c>
+      <c r="Y35">
+        <v>0</v>
+      </c>
+      <c r="Z35">
+        <v>0</v>
+      </c>
+      <c r="AA35">
+        <v>0</v>
+      </c>
+      <c r="AB35">
+        <v>0</v>
+      </c>
+      <c r="AC35">
+        <v>1.89</v>
+      </c>
+      <c r="AD35">
+        <v>1.22</v>
+      </c>
+      <c r="AE35">
+        <v>1.44</v>
+      </c>
+      <c r="AF35">
+        <v>4.75</v>
+      </c>
+      <c r="AG35">
+        <v>6.5</v>
+      </c>
+      <c r="AH35">
+        <v>1.49</v>
+      </c>
+      <c r="AI35">
+        <v>5</v>
+      </c>
+      <c r="AJ35">
+        <v>7.6</v>
+      </c>
+      <c r="AK35">
+        <v>1.53</v>
+      </c>
+      <c r="AL35">
+        <v>4.8</v>
+      </c>
+      <c r="AM35">
+        <v>7.1</v>
+      </c>
+      <c r="AN35">
+        <v>1.46</v>
+      </c>
+      <c r="AO35">
+        <v>4.6500000000000004</v>
+      </c>
+      <c r="AP35">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>266</v>
+      </c>
+      <c r="B36" t="s">
+        <v>135</v>
+      </c>
+      <c r="C36" t="s">
+        <v>27</v>
+      </c>
+      <c r="D36" s="1">
+        <v>46194</v>
+      </c>
+      <c r="E36" s="7">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+      <c r="P36" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q36">
+        <v>27</v>
+      </c>
+      <c r="R36">
+        <v>10</v>
+      </c>
+      <c r="S36">
+        <v>15</v>
+      </c>
+      <c r="T36">
+        <v>3</v>
+      </c>
+      <c r="U36">
+        <v>7</v>
+      </c>
+      <c r="V36">
+        <v>10</v>
+      </c>
+      <c r="W36">
+        <v>9</v>
+      </c>
+      <c r="X36">
+        <v>0</v>
+      </c>
+      <c r="Y36">
+        <v>1</v>
+      </c>
+      <c r="Z36">
+        <v>5</v>
+      </c>
+      <c r="AA36">
+        <v>0</v>
+      </c>
+      <c r="AB36">
+        <v>0</v>
+      </c>
+      <c r="AC36">
+        <v>2.84</v>
+      </c>
+      <c r="AD36">
+        <v>0.5</v>
+      </c>
+      <c r="AE36">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="AF36">
+        <v>9</v>
+      </c>
+      <c r="AG36">
+        <v>15</v>
+      </c>
+      <c r="AH36">
+        <v>1.18</v>
+      </c>
+      <c r="AI36">
+        <v>10</v>
+      </c>
+      <c r="AJ36">
+        <v>18</v>
+      </c>
+      <c r="AK36">
+        <v>1.17</v>
+      </c>
+      <c r="AL36">
+        <v>9.5</v>
+      </c>
+      <c r="AM36">
+        <v>20</v>
+      </c>
+      <c r="AN36">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="AO36">
+        <v>8.15</v>
+      </c>
+      <c r="AP36">
+        <v>16.47</v>
+      </c>
+    </row>
+    <row r="37" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>266</v>
+      </c>
+      <c r="B37" t="s">
+        <v>107</v>
+      </c>
+      <c r="C37" t="s">
+        <v>160</v>
+      </c>
+      <c r="D37" s="1">
+        <v>46194</v>
+      </c>
+      <c r="E37" s="7">
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+      <c r="G37">
+        <v>4</v>
+      </c>
+      <c r="H37">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>2</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
+        <v>2</v>
+      </c>
+      <c r="P37" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q37">
+        <v>2</v>
+      </c>
+      <c r="R37">
+        <v>11</v>
+      </c>
+      <c r="S37">
+        <v>0</v>
+      </c>
+      <c r="T37">
+        <v>5</v>
+      </c>
+      <c r="U37">
+        <v>8</v>
+      </c>
+      <c r="V37">
+        <v>15</v>
+      </c>
+      <c r="W37">
+        <v>3</v>
+      </c>
+      <c r="X37">
+        <v>5</v>
+      </c>
+      <c r="Y37">
+        <v>0</v>
+      </c>
+      <c r="Z37">
+        <v>0</v>
+      </c>
+      <c r="AA37">
+        <v>0</v>
+      </c>
+      <c r="AB37">
+        <v>0</v>
+      </c>
+      <c r="AC37">
+        <v>0.04</v>
+      </c>
+      <c r="AD37">
+        <v>2.13</v>
+      </c>
+      <c r="AE37">
+        <v>8.5</v>
+      </c>
+      <c r="AF37">
+        <v>4.5</v>
+      </c>
+      <c r="AG37">
+        <v>1.4</v>
+      </c>
+      <c r="AH37">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="AI37">
+        <v>4.5</v>
+      </c>
+      <c r="AJ37">
+        <v>1.48</v>
+      </c>
+      <c r="AK37">
+        <v>8.5</v>
+      </c>
+      <c r="AL37">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="AM37">
+        <v>1.48</v>
+      </c>
+      <c r="AN37">
+        <v>7.69</v>
+      </c>
+      <c r="AO37">
+        <v>4.3</v>
+      </c>
+      <c r="AP37">
+        <v>1.43</v>
+      </c>
+    </row>
+    <row r="38" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>266</v>
+      </c>
+      <c r="B38" t="s">
+        <v>44</v>
+      </c>
+      <c r="C38" t="s">
+        <v>83</v>
+      </c>
+      <c r="D38" s="1">
+        <v>46194</v>
+      </c>
+      <c r="E38" s="7">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F38">
+        <v>4</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38">
+        <v>3</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>1</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+      <c r="P38" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q38">
+        <v>22</v>
+      </c>
+      <c r="R38">
+        <v>3</v>
+      </c>
+      <c r="S38">
+        <v>8</v>
+      </c>
+      <c r="T38">
+        <v>1</v>
+      </c>
+      <c r="U38">
+        <v>10</v>
+      </c>
+      <c r="V38">
+        <v>2</v>
+      </c>
+      <c r="W38">
+        <v>6</v>
+      </c>
+      <c r="X38">
+        <v>1</v>
+      </c>
+      <c r="Y38">
+        <v>0</v>
+      </c>
+      <c r="Z38">
+        <v>2</v>
+      </c>
+      <c r="AA38">
+        <v>0</v>
+      </c>
+      <c r="AB38">
+        <v>0</v>
+      </c>
+      <c r="AC38">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AD38">
+        <v>0.13</v>
+      </c>
+      <c r="AE38">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AF38">
+        <v>11</v>
+      </c>
+      <c r="AG38">
+        <v>21</v>
+      </c>
+      <c r="AH38">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="AI38">
+        <v>13</v>
+      </c>
+      <c r="AJ38">
+        <v>28</v>
+      </c>
+      <c r="AK38">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="AL38">
+        <v>13</v>
+      </c>
+      <c r="AM38">
+        <v>27</v>
+      </c>
+      <c r="AN38">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="AO38">
+        <v>10.69</v>
+      </c>
+      <c r="AP38">
+        <v>22.81</v>
+      </c>
+    </row>
+    <row r="39" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>266</v>
+      </c>
+      <c r="B39" t="s">
+        <v>36</v>
+      </c>
+      <c r="C39" t="s">
+        <v>152</v>
+      </c>
+      <c r="D39" s="1">
+        <v>46194</v>
+      </c>
+      <c r="E39" s="7">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39">
+        <v>0</v>
+      </c>
+      <c r="H39">
+        <v>0</v>
+      </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
+      <c r="P39" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q39">
+        <v>23</v>
+      </c>
+      <c r="R39">
+        <v>7</v>
+      </c>
+      <c r="S39">
+        <v>7</v>
+      </c>
+      <c r="T39">
+        <v>3</v>
+      </c>
+      <c r="U39">
+        <v>7</v>
+      </c>
+      <c r="V39">
+        <v>9</v>
+      </c>
+      <c r="W39">
+        <v>4</v>
+      </c>
+      <c r="X39">
+        <v>2</v>
+      </c>
+      <c r="Y39">
+        <v>1</v>
+      </c>
+      <c r="Z39">
+        <v>1</v>
+      </c>
+      <c r="AA39">
+        <v>1</v>
+      </c>
+      <c r="AB39">
+        <v>0</v>
+      </c>
+      <c r="AC39">
+        <v>1.79</v>
+      </c>
+      <c r="AD39">
+        <v>0.62</v>
+      </c>
+      <c r="AE39">
+        <v>1.42</v>
+      </c>
+      <c r="AF39">
+        <v>4.5</v>
+      </c>
+      <c r="AG39">
+        <v>8</v>
+      </c>
+      <c r="AH39">
+        <v>1.45</v>
+      </c>
+      <c r="AI39">
+        <v>4.8</v>
+      </c>
+      <c r="AJ39">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="AK39">
+        <v>1.44</v>
+      </c>
+      <c r="AL39">
+        <v>4.8</v>
+      </c>
+      <c r="AM39">
+        <v>8.5</v>
+      </c>
+      <c r="AN39">
+        <v>1.4</v>
+      </c>
+      <c r="AO39">
+        <v>4.53</v>
+      </c>
+      <c r="AP39">
+        <v>7.87</v>
+      </c>
+    </row>
+    <row r="40" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>266</v>
+      </c>
+      <c r="B40" t="s">
+        <v>130</v>
+      </c>
+      <c r="C40" t="s">
+        <v>97</v>
+      </c>
+      <c r="D40" s="1">
+        <v>46194</v>
+      </c>
+      <c r="E40" s="7">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="F40">
+        <v>2</v>
+      </c>
+      <c r="G40">
+        <v>2</v>
+      </c>
+      <c r="H40">
+        <v>2</v>
+      </c>
+      <c r="I40">
+        <v>1</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <v>1</v>
+      </c>
+      <c r="P40" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q40">
+        <v>17</v>
+      </c>
+      <c r="R40">
+        <v>12</v>
+      </c>
+      <c r="S40">
+        <v>2</v>
+      </c>
+      <c r="T40">
+        <v>4</v>
+      </c>
+      <c r="U40">
+        <v>11</v>
+      </c>
+      <c r="V40">
+        <v>4</v>
+      </c>
+      <c r="W40">
+        <v>11</v>
+      </c>
+      <c r="X40">
+        <v>4</v>
+      </c>
+      <c r="Y40">
+        <v>2</v>
+      </c>
+      <c r="Z40">
+        <v>2</v>
+      </c>
+      <c r="AA40">
+        <v>0</v>
+      </c>
+      <c r="AB40">
+        <v>0</v>
+      </c>
+      <c r="AC40">
+        <v>2.31</v>
+      </c>
+      <c r="AD40">
+        <v>0.88</v>
+      </c>
+      <c r="AE40">
+        <v>1.38</v>
+      </c>
+      <c r="AF40">
+        <v>4.75</v>
+      </c>
+      <c r="AG40">
+        <v>8.5</v>
+      </c>
+      <c r="AH40">
+        <v>1.41</v>
+      </c>
+      <c r="AI40">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="AJ40">
+        <v>11</v>
+      </c>
+      <c r="AK40">
+        <v>1.41</v>
+      </c>
+      <c r="AL40">
+        <v>5</v>
+      </c>
+      <c r="AM40">
+        <v>10</v>
+      </c>
+      <c r="AN40">
+        <v>1.37</v>
+      </c>
+      <c r="AO40">
+        <v>4.5</v>
+      </c>
+      <c r="AP40">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>266</v>
+      </c>
+      <c r="B41" t="s">
+        <v>167</v>
+      </c>
+      <c r="C41" t="s">
+        <v>117</v>
+      </c>
+      <c r="D41" s="1">
+        <v>46195</v>
+      </c>
+      <c r="E41" s="7">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="F41">
+        <v>1</v>
+      </c>
+      <c r="G41">
+        <v>3</v>
+      </c>
+      <c r="H41">
+        <v>1</v>
+      </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41">
+        <v>3</v>
+      </c>
+      <c r="P41" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q41">
+        <v>11</v>
+      </c>
+      <c r="R41">
+        <v>19</v>
+      </c>
+      <c r="S41">
+        <v>5</v>
+      </c>
+      <c r="T41">
+        <v>7</v>
+      </c>
+      <c r="U41">
+        <v>14</v>
+      </c>
+      <c r="V41">
+        <v>8</v>
+      </c>
+      <c r="W41">
+        <v>4</v>
+      </c>
+      <c r="X41">
+        <v>3</v>
+      </c>
+      <c r="Y41">
+        <v>2</v>
+      </c>
+      <c r="Z41">
+        <v>1</v>
+      </c>
+      <c r="AA41">
+        <v>0</v>
+      </c>
+      <c r="AB41">
+        <v>0</v>
+      </c>
+      <c r="AC41">
+        <v>1.24</v>
+      </c>
+      <c r="AD41">
+        <v>1.87</v>
+      </c>
+      <c r="AE41">
+        <v>5.75</v>
+      </c>
+      <c r="AF41">
+        <v>3.9</v>
+      </c>
+      <c r="AG41">
+        <v>1.62</v>
+      </c>
+      <c r="AH41">
+        <v>6.2</v>
+      </c>
+      <c r="AI41">
+        <v>4</v>
+      </c>
+      <c r="AJ41">
+        <v>1.68</v>
+      </c>
+      <c r="AK41">
+        <v>6</v>
+      </c>
+      <c r="AL41">
+        <v>4</v>
+      </c>
+      <c r="AM41">
+        <v>1.67</v>
+      </c>
+      <c r="AN41">
+        <v>5.64</v>
+      </c>
+      <c r="AO41">
+        <v>3.76</v>
+      </c>
+      <c r="AP41">
+        <v>1.61</v>
+      </c>
+    </row>
+    <row r="42" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>266</v>
+      </c>
+      <c r="B42" t="s">
+        <v>136</v>
+      </c>
+      <c r="C42" t="s">
+        <v>33</v>
+      </c>
+      <c r="D42" s="1">
+        <v>46195</v>
+      </c>
+      <c r="E42" s="7">
+        <v>0.75</v>
+      </c>
+      <c r="F42">
+        <v>2</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42">
+        <v>1</v>
+      </c>
+      <c r="I42">
+        <v>0</v>
+      </c>
+      <c r="J42">
+        <v>1</v>
+      </c>
+      <c r="K42">
+        <v>0</v>
+      </c>
+      <c r="P42" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q42">
+        <v>12</v>
+      </c>
+      <c r="R42">
+        <v>6</v>
+      </c>
+      <c r="S42">
+        <v>5</v>
+      </c>
+      <c r="T42">
+        <v>1</v>
+      </c>
+      <c r="U42">
+        <v>13</v>
+      </c>
+      <c r="V42">
+        <v>13</v>
+      </c>
+      <c r="W42">
+        <v>1</v>
+      </c>
+      <c r="X42">
+        <v>3</v>
+      </c>
+      <c r="Y42">
+        <v>2</v>
+      </c>
+      <c r="Z42">
+        <v>2</v>
+      </c>
+      <c r="AA42">
+        <v>0</v>
+      </c>
+      <c r="AB42">
+        <v>0</v>
+      </c>
+      <c r="AC42">
+        <v>2.36</v>
+      </c>
+      <c r="AD42">
+        <v>0.53</v>
+      </c>
+      <c r="AE42">
+        <v>1.44</v>
+      </c>
+      <c r="AF42">
+        <v>4.33</v>
+      </c>
+      <c r="AG42">
+        <v>7.5</v>
+      </c>
+      <c r="AH42">
+        <v>1.49</v>
+      </c>
+      <c r="AI42">
+        <v>4.5</v>
+      </c>
+      <c r="AJ42">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="AK42">
+        <v>1.48</v>
+      </c>
+      <c r="AL42">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="AM42">
+        <v>8</v>
+      </c>
+      <c r="AN42">
+        <v>1.44</v>
+      </c>
+      <c r="AO42">
+        <v>4.33</v>
+      </c>
+      <c r="AP42">
+        <v>7.32</v>
+      </c>
+    </row>
+    <row r="43" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>266</v>
+      </c>
+      <c r="B43" t="s">
+        <v>60</v>
+      </c>
+      <c r="C43" t="s">
+        <v>1</v>
+      </c>
+      <c r="D43" s="1">
+        <v>46195</v>
+      </c>
+      <c r="E43" s="7">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="F43">
+        <v>3</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43">
+        <v>1</v>
+      </c>
+      <c r="I43">
+        <v>0</v>
+      </c>
+      <c r="J43">
+        <v>2</v>
+      </c>
+      <c r="K43">
+        <v>0</v>
+      </c>
+      <c r="P43" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q43">
+        <v>19</v>
+      </c>
+      <c r="R43">
+        <v>4</v>
+      </c>
+      <c r="S43">
+        <v>5</v>
+      </c>
+      <c r="T43">
+        <v>0</v>
+      </c>
+      <c r="U43">
+        <v>8</v>
+      </c>
+      <c r="V43">
+        <v>4</v>
+      </c>
+      <c r="W43">
+        <v>4</v>
+      </c>
+      <c r="X43">
+        <v>2</v>
+      </c>
+      <c r="Y43">
+        <v>0</v>
+      </c>
+      <c r="Z43">
+        <v>1</v>
+      </c>
+      <c r="AA43">
+        <v>0</v>
+      </c>
+      <c r="AB43">
+        <v>0</v>
+      </c>
+      <c r="AC43">
+        <v>2.67</v>
+      </c>
+      <c r="AD43">
+        <v>0.62</v>
+      </c>
+      <c r="AE43">
+        <v>1.07</v>
+      </c>
+      <c r="AF43">
+        <v>12</v>
+      </c>
+      <c r="AG43">
+        <v>26</v>
+      </c>
+      <c r="AH43">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="AI43">
+        <v>15</v>
+      </c>
+      <c r="AJ43">
+        <v>48</v>
+      </c>
+      <c r="AK43">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="AL43">
+        <v>14</v>
+      </c>
+      <c r="AM43">
+        <v>36</v>
+      </c>
+      <c r="AN43">
+        <v>1.07</v>
+      </c>
+      <c r="AO43">
+        <v>12.03</v>
+      </c>
+      <c r="AP43">
+        <v>28.13</v>
+      </c>
+    </row>
+    <row r="44" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>266</v>
+      </c>
+      <c r="B44" t="s">
+        <v>56</v>
+      </c>
+      <c r="C44" t="s">
+        <v>81</v>
+      </c>
+      <c r="D44" s="1">
+        <v>46196</v>
+      </c>
+      <c r="E44" s="7">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F44">
+        <v>3</v>
+      </c>
+      <c r="G44">
+        <v>2</v>
+      </c>
+      <c r="H44">
+        <v>1</v>
+      </c>
+      <c r="I44">
+        <v>0</v>
+      </c>
+      <c r="J44">
+        <v>2</v>
+      </c>
+      <c r="K44">
+        <v>2</v>
+      </c>
+      <c r="P44" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q44">
+        <v>13</v>
+      </c>
+      <c r="R44">
+        <v>16</v>
+      </c>
+      <c r="S44">
+        <v>7</v>
+      </c>
+      <c r="T44">
+        <v>4</v>
+      </c>
+      <c r="U44">
+        <v>13</v>
+      </c>
+      <c r="V44">
+        <v>5</v>
+      </c>
+      <c r="W44">
+        <v>5</v>
+      </c>
+      <c r="X44">
+        <v>4</v>
+      </c>
+      <c r="Y44">
+        <v>0</v>
+      </c>
+      <c r="Z44">
+        <v>0</v>
+      </c>
+      <c r="AA44">
+        <v>0</v>
+      </c>
+      <c r="AB44">
+        <v>0</v>
+      </c>
+      <c r="AC44">
+        <v>2.19</v>
+      </c>
+      <c r="AD44">
+        <v>1.71</v>
+      </c>
+      <c r="AE44">
+        <v>2.4</v>
+      </c>
+      <c r="AF44">
+        <v>3.5</v>
+      </c>
+      <c r="AG44">
+        <v>2.88</v>
+      </c>
+      <c r="AH44">
+        <v>2.6</v>
+      </c>
+      <c r="AI44">
+        <v>3.5</v>
+      </c>
+      <c r="AJ44">
+        <v>3</v>
+      </c>
+      <c r="AK44">
+        <v>2.5</v>
+      </c>
+      <c r="AL44">
+        <v>3.5</v>
+      </c>
+      <c r="AM44">
+        <v>3.05</v>
+      </c>
+      <c r="AN44">
+        <v>2.39</v>
+      </c>
+      <c r="AO44">
+        <v>3.39</v>
+      </c>
+      <c r="AP44">
+        <v>2.85</v>
+      </c>
+    </row>
+    <row r="45" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>266</v>
+      </c>
+      <c r="B45" t="s">
+        <v>150</v>
+      </c>
+      <c r="C45" t="s">
+        <v>87</v>
+      </c>
+      <c r="D45" s="1">
+        <v>46196</v>
+      </c>
+      <c r="E45" s="7">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="F45">
+        <v>1</v>
+      </c>
+      <c r="G45">
+        <v>2</v>
+      </c>
+      <c r="H45">
+        <v>1</v>
+      </c>
+      <c r="I45">
+        <v>0</v>
+      </c>
+      <c r="J45">
+        <v>0</v>
+      </c>
+      <c r="K45">
+        <v>2</v>
+      </c>
+      <c r="P45" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q45">
+        <v>8</v>
+      </c>
+      <c r="R45">
+        <v>17</v>
+      </c>
+      <c r="S45">
+        <v>4</v>
+      </c>
+      <c r="T45">
+        <v>8</v>
+      </c>
+      <c r="U45">
+        <v>11</v>
+      </c>
+      <c r="V45">
+        <v>6</v>
+      </c>
+      <c r="W45">
+        <v>1</v>
+      </c>
+      <c r="X45">
+        <v>10</v>
+      </c>
+      <c r="Y45">
+        <v>1</v>
+      </c>
+      <c r="Z45">
+        <v>1</v>
+      </c>
+      <c r="AA45">
+        <v>0</v>
+      </c>
+      <c r="AB45">
+        <v>0</v>
+      </c>
+      <c r="AC45">
+        <v>0.64</v>
+      </c>
+      <c r="AD45">
+        <v>1.89</v>
+      </c>
+      <c r="AE45">
+        <v>7</v>
+      </c>
+      <c r="AF45">
+        <v>4.5</v>
+      </c>
+      <c r="AG45">
+        <v>1.45</v>
+      </c>
+      <c r="AH45">
+        <v>7.6</v>
+      </c>
+      <c r="AI45">
+        <v>4.7</v>
+      </c>
+      <c r="AJ45">
+        <v>1.51</v>
+      </c>
+      <c r="AK45">
+        <v>7.5</v>
+      </c>
+      <c r="AL45">
+        <v>4.5</v>
+      </c>
+      <c r="AM45">
+        <v>1.53</v>
+      </c>
+      <c r="AN45">
+        <v>6.87</v>
+      </c>
+      <c r="AO45">
+        <v>4.37</v>
+      </c>
+      <c r="AP45">
+        <v>1.46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>266</v>
+      </c>
+      <c r="B46" t="s">
+        <v>64</v>
+      </c>
+      <c r="C46" t="s">
+        <v>155</v>
+      </c>
+      <c r="D46" s="1">
+        <v>46196</v>
+      </c>
+      <c r="E46" s="7">
+        <v>0.75</v>
+      </c>
+      <c r="F46">
+        <v>5</v>
+      </c>
+      <c r="G46">
+        <v>0</v>
+      </c>
+      <c r="H46">
+        <v>3</v>
+      </c>
+      <c r="I46">
+        <v>0</v>
+      </c>
+      <c r="J46">
+        <v>2</v>
+      </c>
+      <c r="K46">
+        <v>0</v>
+      </c>
+      <c r="P46" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q46">
+        <v>17</v>
+      </c>
+      <c r="R46">
+        <v>7</v>
+      </c>
+      <c r="S46">
+        <v>9</v>
+      </c>
+      <c r="T46">
+        <v>2</v>
+      </c>
+      <c r="U46">
+        <v>14</v>
+      </c>
+      <c r="V46">
+        <v>15</v>
+      </c>
+      <c r="W46">
+        <v>3</v>
+      </c>
+      <c r="X46">
+        <v>2</v>
+      </c>
+      <c r="Y46">
+        <v>1</v>
+      </c>
+      <c r="Z46">
+        <v>1</v>
+      </c>
+      <c r="AA46">
+        <v>0</v>
+      </c>
+      <c r="AB46">
+        <v>0</v>
+      </c>
+      <c r="AC46">
+        <v>2.6</v>
+      </c>
+      <c r="AD46">
+        <v>0.25</v>
+      </c>
+      <c r="AE46">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="AF46">
+        <v>9</v>
+      </c>
+      <c r="AG46">
+        <v>19</v>
+      </c>
+      <c r="AH46">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="AI46">
+        <v>9.6</v>
+      </c>
+      <c r="AJ46">
+        <v>25</v>
+      </c>
+      <c r="AK46">
+        <v>1.17</v>
+      </c>
+      <c r="AL46">
+        <v>9</v>
+      </c>
+      <c r="AM46">
+        <v>22</v>
+      </c>
+      <c r="AN46">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="AO46">
+        <v>8.48</v>
+      </c>
+      <c r="AP46">
+        <v>19.309999999999999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>266</v>
+      </c>
+      <c r="B47" t="s">
+        <v>58</v>
+      </c>
+      <c r="C47" t="s">
+        <v>113</v>
+      </c>
+      <c r="D47" s="1">
+        <v>46196</v>
+      </c>
+      <c r="E47" s="7">
+        <v>0.875</v>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47">
+        <v>0</v>
+      </c>
+      <c r="H47">
+        <v>0</v>
+      </c>
+      <c r="I47">
+        <v>0</v>
+      </c>
+      <c r="J47">
+        <v>0</v>
+      </c>
+      <c r="K47">
+        <v>0</v>
+      </c>
+      <c r="P47" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q47">
+        <v>19</v>
+      </c>
+      <c r="R47">
+        <v>2</v>
+      </c>
+      <c r="S47">
+        <v>3</v>
+      </c>
+      <c r="T47">
+        <v>1</v>
+      </c>
+      <c r="U47">
+        <v>14</v>
+      </c>
+      <c r="V47">
+        <v>24</v>
+      </c>
+      <c r="W47">
+        <v>9</v>
+      </c>
+      <c r="X47">
+        <v>2</v>
+      </c>
+      <c r="Y47">
+        <v>1</v>
+      </c>
+      <c r="Z47">
+        <v>1</v>
+      </c>
+      <c r="AA47">
+        <v>0</v>
+      </c>
+      <c r="AB47">
+        <v>0</v>
+      </c>
+      <c r="AC47">
+        <v>1.36</v>
+      </c>
+      <c r="AD47">
+        <v>0.17</v>
+      </c>
+      <c r="AE47">
+        <v>1.18</v>
+      </c>
+      <c r="AF47">
+        <v>7.5</v>
+      </c>
+      <c r="AG47">
+        <v>15</v>
+      </c>
+      <c r="AH47">
+        <v>1.2</v>
+      </c>
+      <c r="AI47">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="AJ47">
+        <v>21</v>
+      </c>
+      <c r="AK47">
+        <v>1.2</v>
+      </c>
+      <c r="AL47">
+        <v>8</v>
+      </c>
+      <c r="AM47">
+        <v>19</v>
+      </c>
+      <c r="AN47">
+        <v>1.17</v>
+      </c>
+      <c r="AO47">
+        <v>7.29</v>
+      </c>
+      <c r="AP47">
+        <v>15.28</v>
+      </c>
+    </row>
+    <row r="48" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>266</v>
+      </c>
+      <c r="B48" t="s">
+        <v>28</v>
+      </c>
+      <c r="C48" t="s">
+        <v>47</v>
+      </c>
+      <c r="D48" s="1">
+        <v>46197</v>
+      </c>
+      <c r="E48" s="7">
+        <v>0</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+      <c r="G48">
+        <v>1</v>
+      </c>
+      <c r="H48">
+        <v>0</v>
+      </c>
+      <c r="I48">
+        <v>0</v>
+      </c>
+      <c r="J48">
+        <v>0</v>
+      </c>
+      <c r="K48">
+        <v>1</v>
+      </c>
+      <c r="P48" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q48">
+        <v>8</v>
+      </c>
+      <c r="R48">
+        <v>6</v>
+      </c>
+      <c r="S48">
+        <v>1</v>
+      </c>
+      <c r="T48">
+        <v>2</v>
+      </c>
+      <c r="U48">
+        <v>19</v>
+      </c>
+      <c r="V48">
+        <v>12</v>
+      </c>
+      <c r="W48">
+        <v>7</v>
+      </c>
+      <c r="X48">
+        <v>2</v>
+      </c>
+      <c r="Y48">
+        <v>1</v>
+      </c>
+      <c r="Z48">
+        <v>1</v>
+      </c>
+      <c r="AA48">
+        <v>0</v>
+      </c>
+      <c r="AB48">
+        <v>0</v>
+      </c>
+      <c r="AC48">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AD48">
+        <v>1.65</v>
+      </c>
+      <c r="AE48">
+        <v>7.5</v>
+      </c>
+      <c r="AF48">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="AG48">
+        <v>1.42</v>
+      </c>
+      <c r="AH48">
+        <v>9</v>
+      </c>
+      <c r="AI48">
+        <v>4.8</v>
+      </c>
+      <c r="AJ48">
+        <v>1.45</v>
+      </c>
+      <c r="AK48">
+        <v>8</v>
+      </c>
+      <c r="AL48">
+        <v>4.8</v>
+      </c>
+      <c r="AM48">
+        <v>1.44</v>
+      </c>
+      <c r="AN48">
+        <v>7.82</v>
+      </c>
+      <c r="AO48">
+        <v>4.55</v>
+      </c>
+      <c r="AP48">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>266</v>
+      </c>
+      <c r="B49" t="s">
+        <v>132</v>
+      </c>
+      <c r="C49" t="s">
+        <v>3</v>
+      </c>
+      <c r="D49" s="1">
+        <v>46197</v>
+      </c>
+      <c r="E49" s="7">
+        <v>0.125</v>
+      </c>
+      <c r="F49">
+        <v>1</v>
+      </c>
+      <c r="G49">
+        <v>0</v>
+      </c>
+      <c r="H49">
+        <v>0</v>
+      </c>
+      <c r="I49">
+        <v>0</v>
+      </c>
+      <c r="J49">
+        <v>1</v>
+      </c>
+      <c r="K49">
+        <v>0</v>
+      </c>
+      <c r="P49" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q49">
+        <v>20</v>
+      </c>
+      <c r="R49">
+        <v>7</v>
+      </c>
+      <c r="S49">
+        <v>9</v>
+      </c>
+      <c r="T49">
+        <v>1</v>
+      </c>
+      <c r="U49">
+        <v>12</v>
+      </c>
+      <c r="V49">
+        <v>16</v>
+      </c>
+      <c r="W49">
+        <v>5</v>
+      </c>
+      <c r="X49">
+        <v>4</v>
+      </c>
+      <c r="Y49">
+        <v>2</v>
+      </c>
+      <c r="Z49">
+        <v>1</v>
+      </c>
+      <c r="AA49">
+        <v>0</v>
+      </c>
+      <c r="AB49">
+        <v>0</v>
+      </c>
+      <c r="AC49">
+        <v>0.98</v>
+      </c>
+      <c r="AD49">
+        <v>0.37</v>
+      </c>
+      <c r="AE49">
+        <v>1.53</v>
+      </c>
+      <c r="AF49">
+        <v>3.9</v>
+      </c>
+      <c r="AG49">
+        <v>7</v>
+      </c>
+      <c r="AH49">
+        <v>1.56</v>
+      </c>
+      <c r="AI49">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AJ49">
+        <v>8</v>
+      </c>
+      <c r="AK49">
+        <v>1.55</v>
+      </c>
+      <c r="AL49">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AM49">
+        <v>7.1</v>
+      </c>
+      <c r="AN49">
+        <v>1.52</v>
+      </c>
+      <c r="AO49">
+        <v>3.93</v>
+      </c>
+      <c r="AP49">
+        <v>6.71</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AP25">
-    <sortCondition ref="D2:D25"/>
-    <sortCondition ref="E2:E25"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AP49">
+    <sortCondition ref="D2:D49"/>
+    <sortCondition ref="E2:E49"/>
   </sortState>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
added new xlsx sheet updated with all of completed groupstage matches (as of 28/06/26)
</commit_message>
<xml_diff>
--- a/data/WorldCup2026.xlsx
+++ b/data/WorldCup2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ee16c21b72f3fde9/Documents/Football Fortunes/All data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="170" documentId="8_{9D3D8A05-EEFD-4F90-A3C5-55C1E757FCE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95330EEB-27A4-410B-8772-81AD9AFCF4C8}"/>
+  <xr:revisionPtr revIDLastSave="176" documentId="8_{9D3D8A05-EEFD-4F90-A3C5-55C1E757FCE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EFAAA261-4024-4339-887D-3A027308D725}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{95D741F4-B12C-45C7-A97C-F95A56A544CF}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2928" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3024" uniqueCount="267">
   <si>
     <t>Home</t>
   </si>
@@ -1235,7 +1235,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73F33CE9-0917-4340-92ED-8B6CE132D95A}">
-  <dimension ref="A1:AP49"/>
+  <dimension ref="A1:AP73"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.54296875" bestFit="1" customWidth="1"/>
@@ -6969,10 +6969,2794 @@
         <v>6.71</v>
       </c>
     </row>
+    <row r="50" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>266</v>
+      </c>
+      <c r="B50" t="s">
+        <v>5</v>
+      </c>
+      <c r="C50" t="s">
+        <v>84</v>
+      </c>
+      <c r="D50" s="1">
+        <v>46197</v>
+      </c>
+      <c r="E50" s="7">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F50">
+        <v>3</v>
+      </c>
+      <c r="G50">
+        <v>1</v>
+      </c>
+      <c r="H50">
+        <v>2</v>
+      </c>
+      <c r="I50">
+        <v>1</v>
+      </c>
+      <c r="J50">
+        <v>1</v>
+      </c>
+      <c r="K50">
+        <v>0</v>
+      </c>
+      <c r="P50" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q50">
+        <v>14</v>
+      </c>
+      <c r="R50">
+        <v>9</v>
+      </c>
+      <c r="S50">
+        <v>5</v>
+      </c>
+      <c r="T50">
+        <v>3</v>
+      </c>
+      <c r="U50">
+        <v>9</v>
+      </c>
+      <c r="V50">
+        <v>14</v>
+      </c>
+      <c r="W50">
+        <v>5</v>
+      </c>
+      <c r="X50">
+        <v>5</v>
+      </c>
+      <c r="Y50">
+        <v>1</v>
+      </c>
+      <c r="Z50">
+        <v>1</v>
+      </c>
+      <c r="AA50">
+        <v>0</v>
+      </c>
+      <c r="AB50">
+        <v>0</v>
+      </c>
+      <c r="AC50">
+        <v>0.68</v>
+      </c>
+      <c r="AD50">
+        <v>0.77</v>
+      </c>
+      <c r="AE50">
+        <v>1.4</v>
+      </c>
+      <c r="AF50">
+        <v>5</v>
+      </c>
+      <c r="AG50">
+        <v>7</v>
+      </c>
+      <c r="AH50">
+        <v>1.45</v>
+      </c>
+      <c r="AI50">
+        <v>5.2</v>
+      </c>
+      <c r="AJ50">
+        <v>8</v>
+      </c>
+      <c r="AK50">
+        <v>1.45</v>
+      </c>
+      <c r="AL50">
+        <v>5.2</v>
+      </c>
+      <c r="AM50">
+        <v>8</v>
+      </c>
+      <c r="AN50">
+        <v>1.4</v>
+      </c>
+      <c r="AO50">
+        <v>4.87</v>
+      </c>
+      <c r="AP50">
+        <v>7.02</v>
+      </c>
+    </row>
+    <row r="51" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>266</v>
+      </c>
+      <c r="B51" t="s">
+        <v>41</v>
+      </c>
+      <c r="C51" t="s">
+        <v>258</v>
+      </c>
+      <c r="D51" s="1">
+        <v>46197</v>
+      </c>
+      <c r="E51" s="7">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F51">
+        <v>2</v>
+      </c>
+      <c r="G51">
+        <v>1</v>
+      </c>
+      <c r="H51">
+        <v>0</v>
+      </c>
+      <c r="I51">
+        <v>0</v>
+      </c>
+      <c r="J51">
+        <v>2</v>
+      </c>
+      <c r="K51">
+        <v>1</v>
+      </c>
+      <c r="P51" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q51">
+        <v>6</v>
+      </c>
+      <c r="R51">
+        <v>13</v>
+      </c>
+      <c r="S51">
+        <v>4</v>
+      </c>
+      <c r="T51">
+        <v>7</v>
+      </c>
+      <c r="U51">
+        <v>19</v>
+      </c>
+      <c r="V51">
+        <v>13</v>
+      </c>
+      <c r="W51">
+        <v>2</v>
+      </c>
+      <c r="X51">
+        <v>7</v>
+      </c>
+      <c r="Y51">
+        <v>1</v>
+      </c>
+      <c r="Z51">
+        <v>2</v>
+      </c>
+      <c r="AA51">
+        <v>0</v>
+      </c>
+      <c r="AB51">
+        <v>0</v>
+      </c>
+      <c r="AC51">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="AD51">
+        <v>1.66</v>
+      </c>
+      <c r="AE51">
+        <v>2.6</v>
+      </c>
+      <c r="AF51">
+        <v>3</v>
+      </c>
+      <c r="AG51">
+        <v>3</v>
+      </c>
+      <c r="AH51">
+        <v>2.7</v>
+      </c>
+      <c r="AI51">
+        <v>3</v>
+      </c>
+      <c r="AJ51">
+        <v>3.3</v>
+      </c>
+      <c r="AK51">
+        <v>2.6</v>
+      </c>
+      <c r="AL51">
+        <v>3.1</v>
+      </c>
+      <c r="AM51">
+        <v>3.25</v>
+      </c>
+      <c r="AN51">
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="AO51">
+        <v>2.95</v>
+      </c>
+      <c r="AP51">
+        <v>3.11</v>
+      </c>
+    </row>
+    <row r="52" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>266</v>
+      </c>
+      <c r="B52" t="s">
+        <v>76</v>
+      </c>
+      <c r="C52" t="s">
+        <v>31</v>
+      </c>
+      <c r="D52" s="1">
+        <v>46197</v>
+      </c>
+      <c r="E52" s="7">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="F52">
+        <v>4</v>
+      </c>
+      <c r="G52">
+        <v>2</v>
+      </c>
+      <c r="H52">
+        <v>2</v>
+      </c>
+      <c r="I52">
+        <v>2</v>
+      </c>
+      <c r="J52">
+        <v>2</v>
+      </c>
+      <c r="K52">
+        <v>0</v>
+      </c>
+      <c r="P52" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q52">
+        <v>22</v>
+      </c>
+      <c r="R52">
+        <v>9</v>
+      </c>
+      <c r="S52">
+        <v>11</v>
+      </c>
+      <c r="T52">
+        <v>2</v>
+      </c>
+      <c r="U52">
+        <v>10</v>
+      </c>
+      <c r="V52">
+        <v>18</v>
+      </c>
+      <c r="W52">
+        <v>9</v>
+      </c>
+      <c r="X52">
+        <v>1</v>
+      </c>
+      <c r="Y52">
+        <v>0</v>
+      </c>
+      <c r="Z52">
+        <v>3</v>
+      </c>
+      <c r="AA52">
+        <v>0</v>
+      </c>
+      <c r="AB52">
+        <v>0</v>
+      </c>
+      <c r="AC52">
+        <v>3.76</v>
+      </c>
+      <c r="AD52">
+        <v>1.22</v>
+      </c>
+      <c r="AE52">
+        <v>1.33</v>
+      </c>
+      <c r="AF52">
+        <v>5.5</v>
+      </c>
+      <c r="AG52">
+        <v>9</v>
+      </c>
+      <c r="AH52">
+        <v>1.32</v>
+      </c>
+      <c r="AI52">
+        <v>6</v>
+      </c>
+      <c r="AJ52">
+        <v>12</v>
+      </c>
+      <c r="AK52">
+        <v>1.33</v>
+      </c>
+      <c r="AL52">
+        <v>6.25</v>
+      </c>
+      <c r="AM52">
+        <v>12</v>
+      </c>
+      <c r="AN52">
+        <v>1.28</v>
+      </c>
+      <c r="AO52">
+        <v>5.66</v>
+      </c>
+      <c r="AP52">
+        <v>9.93</v>
+      </c>
+    </row>
+    <row r="53" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>266</v>
+      </c>
+      <c r="B53" t="s">
+        <v>40</v>
+      </c>
+      <c r="C53" t="s">
+        <v>128</v>
+      </c>
+      <c r="D53" s="1">
+        <v>46197</v>
+      </c>
+      <c r="E53" s="7">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="F53">
+        <v>0</v>
+      </c>
+      <c r="G53">
+        <v>3</v>
+      </c>
+      <c r="H53">
+        <v>0</v>
+      </c>
+      <c r="I53">
+        <v>2</v>
+      </c>
+      <c r="J53">
+        <v>0</v>
+      </c>
+      <c r="K53">
+        <v>1</v>
+      </c>
+      <c r="P53" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q53">
+        <v>14</v>
+      </c>
+      <c r="R53">
+        <v>21</v>
+      </c>
+      <c r="S53">
+        <v>5</v>
+      </c>
+      <c r="T53">
+        <v>9</v>
+      </c>
+      <c r="U53">
+        <v>10</v>
+      </c>
+      <c r="V53">
+        <v>11</v>
+      </c>
+      <c r="W53">
+        <v>7</v>
+      </c>
+      <c r="X53">
+        <v>6</v>
+      </c>
+      <c r="Y53">
+        <v>1</v>
+      </c>
+      <c r="Z53">
+        <v>2</v>
+      </c>
+      <c r="AA53">
+        <v>0</v>
+      </c>
+      <c r="AB53">
+        <v>0</v>
+      </c>
+      <c r="AC53">
+        <v>1.05</v>
+      </c>
+      <c r="AD53">
+        <v>4.34</v>
+      </c>
+      <c r="AE53">
+        <v>10</v>
+      </c>
+      <c r="AF53">
+        <v>5.5</v>
+      </c>
+      <c r="AG53">
+        <v>1.29</v>
+      </c>
+      <c r="AH53">
+        <v>11.5</v>
+      </c>
+      <c r="AI53">
+        <v>5.6</v>
+      </c>
+      <c r="AJ53">
+        <v>1.35</v>
+      </c>
+      <c r="AK53">
+        <v>11</v>
+      </c>
+      <c r="AL53">
+        <v>5.75</v>
+      </c>
+      <c r="AM53">
+        <v>1.35</v>
+      </c>
+      <c r="AN53">
+        <v>9.9</v>
+      </c>
+      <c r="AO53">
+        <v>5.28</v>
+      </c>
+      <c r="AP53">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="54" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>266</v>
+      </c>
+      <c r="B54" t="s">
+        <v>7</v>
+      </c>
+      <c r="C54" t="s">
+        <v>253</v>
+      </c>
+      <c r="D54" s="1">
+        <v>46198</v>
+      </c>
+      <c r="E54" s="7">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="F54">
+        <v>0</v>
+      </c>
+      <c r="G54">
+        <v>3</v>
+      </c>
+      <c r="H54">
+        <v>0</v>
+      </c>
+      <c r="I54">
+        <v>0</v>
+      </c>
+      <c r="J54">
+        <v>0</v>
+      </c>
+      <c r="K54">
+        <v>3</v>
+      </c>
+      <c r="P54" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q54">
+        <v>13</v>
+      </c>
+      <c r="R54">
+        <v>11</v>
+      </c>
+      <c r="S54">
+        <v>1</v>
+      </c>
+      <c r="T54">
+        <v>5</v>
+      </c>
+      <c r="U54">
+        <v>9</v>
+      </c>
+      <c r="V54">
+        <v>13</v>
+      </c>
+      <c r="W54">
+        <v>5</v>
+      </c>
+      <c r="X54">
+        <v>1</v>
+      </c>
+      <c r="Y54">
+        <v>0</v>
+      </c>
+      <c r="Z54">
+        <v>1</v>
+      </c>
+      <c r="AA54">
+        <v>0</v>
+      </c>
+      <c r="AB54">
+        <v>0</v>
+      </c>
+      <c r="AC54">
+        <v>0.48</v>
+      </c>
+      <c r="AD54">
+        <v>1.75</v>
+      </c>
+      <c r="AE54">
+        <v>4.2</v>
+      </c>
+      <c r="AF54">
+        <v>3.9</v>
+      </c>
+      <c r="AG54">
+        <v>1.75</v>
+      </c>
+      <c r="AH54">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="AI54">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AJ54">
+        <v>1.79</v>
+      </c>
+      <c r="AK54">
+        <v>4.8499999999999996</v>
+      </c>
+      <c r="AL54">
+        <v>4</v>
+      </c>
+      <c r="AM54">
+        <v>1.77</v>
+      </c>
+      <c r="AN54">
+        <v>4.42</v>
+      </c>
+      <c r="AO54">
+        <v>3.84</v>
+      </c>
+      <c r="AP54">
+        <v>1.73</v>
+      </c>
+    </row>
+    <row r="55" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>266</v>
+      </c>
+      <c r="B55" t="s">
+        <v>85</v>
+      </c>
+      <c r="C55" t="s">
+        <v>158</v>
+      </c>
+      <c r="D55" s="1">
+        <v>46198</v>
+      </c>
+      <c r="E55" s="7">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
+      <c r="G55">
+        <v>0</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55">
+        <v>0</v>
+      </c>
+      <c r="J55">
+        <v>1</v>
+      </c>
+      <c r="K55">
+        <v>0</v>
+      </c>
+      <c r="P55" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q55">
+        <v>13</v>
+      </c>
+      <c r="R55">
+        <v>8</v>
+      </c>
+      <c r="S55">
+        <v>4</v>
+      </c>
+      <c r="T55">
+        <v>3</v>
+      </c>
+      <c r="U55">
+        <v>7</v>
+      </c>
+      <c r="V55">
+        <v>9</v>
+      </c>
+      <c r="W55">
+        <v>4</v>
+      </c>
+      <c r="X55">
+        <v>6</v>
+      </c>
+      <c r="Y55">
+        <v>1</v>
+      </c>
+      <c r="Z55">
+        <v>1</v>
+      </c>
+      <c r="AA55">
+        <v>0</v>
+      </c>
+      <c r="AB55">
+        <v>0</v>
+      </c>
+      <c r="AC55">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="AD55">
+        <v>0.91</v>
+      </c>
+      <c r="AE55">
+        <v>5.25</v>
+      </c>
+      <c r="AF55">
+        <v>3.75</v>
+      </c>
+      <c r="AG55">
+        <v>1.67</v>
+      </c>
+      <c r="AH55">
+        <v>5.8</v>
+      </c>
+      <c r="AI55">
+        <v>3.8</v>
+      </c>
+      <c r="AJ55">
+        <v>1.76</v>
+      </c>
+      <c r="AK55">
+        <v>6</v>
+      </c>
+      <c r="AL55">
+        <v>3.75</v>
+      </c>
+      <c r="AM55">
+        <v>1.7</v>
+      </c>
+      <c r="AN55">
+        <v>5.42</v>
+      </c>
+      <c r="AO55">
+        <v>3.64</v>
+      </c>
+      <c r="AP55">
+        <v>1.66</v>
+      </c>
+    </row>
+    <row r="56" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>266</v>
+      </c>
+      <c r="B56" t="s">
+        <v>27</v>
+      </c>
+      <c r="C56" t="s">
+        <v>79</v>
+      </c>
+      <c r="D56" s="1">
+        <v>46198</v>
+      </c>
+      <c r="E56" s="7">
+        <v>0.875</v>
+      </c>
+      <c r="F56">
+        <v>0</v>
+      </c>
+      <c r="G56">
+        <v>2</v>
+      </c>
+      <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56">
+        <v>1</v>
+      </c>
+      <c r="J56">
+        <v>0</v>
+      </c>
+      <c r="K56">
+        <v>1</v>
+      </c>
+      <c r="P56" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q56">
+        <v>11</v>
+      </c>
+      <c r="R56">
+        <v>7</v>
+      </c>
+      <c r="S56">
+        <v>2</v>
+      </c>
+      <c r="T56">
+        <v>3</v>
+      </c>
+      <c r="U56">
+        <v>11</v>
+      </c>
+      <c r="V56">
+        <v>6</v>
+      </c>
+      <c r="W56">
+        <v>4</v>
+      </c>
+      <c r="X56">
+        <v>6</v>
+      </c>
+      <c r="Y56">
+        <v>2</v>
+      </c>
+      <c r="Z56">
+        <v>1</v>
+      </c>
+      <c r="AA56">
+        <v>0</v>
+      </c>
+      <c r="AB56">
+        <v>0</v>
+      </c>
+      <c r="AC56">
+        <v>0.5</v>
+      </c>
+      <c r="AD56">
+        <v>1.31</v>
+      </c>
+      <c r="AE56">
+        <v>15</v>
+      </c>
+      <c r="AF56">
+        <v>8</v>
+      </c>
+      <c r="AG56">
+        <v>1.17</v>
+      </c>
+      <c r="AH56">
+        <v>18.5</v>
+      </c>
+      <c r="AI56">
+        <v>8.6</v>
+      </c>
+      <c r="AJ56">
+        <v>1.2</v>
+      </c>
+      <c r="AK56">
+        <v>19</v>
+      </c>
+      <c r="AL56">
+        <v>8.25</v>
+      </c>
+      <c r="AM56">
+        <v>1.19</v>
+      </c>
+      <c r="AN56">
+        <v>16.09</v>
+      </c>
+      <c r="AO56">
+        <v>7.72</v>
+      </c>
+      <c r="AP56">
+        <v>1.1599999999999999</v>
+      </c>
+    </row>
+    <row r="57" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>266</v>
+      </c>
+      <c r="B57" t="s">
+        <v>135</v>
+      </c>
+      <c r="C57" t="s">
+        <v>49</v>
+      </c>
+      <c r="D57" s="1">
+        <v>46198</v>
+      </c>
+      <c r="E57" s="7">
+        <v>0.875</v>
+      </c>
+      <c r="F57">
+        <v>2</v>
+      </c>
+      <c r="G57">
+        <v>1</v>
+      </c>
+      <c r="H57">
+        <v>1</v>
+      </c>
+      <c r="I57">
+        <v>1</v>
+      </c>
+      <c r="J57">
+        <v>1</v>
+      </c>
+      <c r="K57">
+        <v>0</v>
+      </c>
+      <c r="P57" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q57">
+        <v>7</v>
+      </c>
+      <c r="R57">
+        <v>11</v>
+      </c>
+      <c r="S57">
+        <v>3</v>
+      </c>
+      <c r="T57">
+        <v>3</v>
+      </c>
+      <c r="U57">
+        <v>15</v>
+      </c>
+      <c r="V57">
+        <v>10</v>
+      </c>
+      <c r="W57">
+        <v>3</v>
+      </c>
+      <c r="X57">
+        <v>2</v>
+      </c>
+      <c r="Y57">
+        <v>3</v>
+      </c>
+      <c r="Z57">
+        <v>1</v>
+      </c>
+      <c r="AA57">
+        <v>0</v>
+      </c>
+      <c r="AB57">
+        <v>0</v>
+      </c>
+      <c r="AC57">
+        <v>1.27</v>
+      </c>
+      <c r="AD57">
+        <v>0.65</v>
+      </c>
+      <c r="AE57">
+        <v>4.33</v>
+      </c>
+      <c r="AF57">
+        <v>4.2</v>
+      </c>
+      <c r="AG57">
+        <v>1.7</v>
+      </c>
+      <c r="AH57">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="AI57">
+        <v>4.5</v>
+      </c>
+      <c r="AJ57">
+        <v>1.77</v>
+      </c>
+      <c r="AK57">
+        <v>4.7</v>
+      </c>
+      <c r="AL57">
+        <v>4.33</v>
+      </c>
+      <c r="AM57">
+        <v>1.75</v>
+      </c>
+      <c r="AN57">
+        <v>4.25</v>
+      </c>
+      <c r="AO57">
+        <v>4.1399999999999997</v>
+      </c>
+      <c r="AP57">
+        <v>1.71</v>
+      </c>
+    </row>
+    <row r="58" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>266</v>
+      </c>
+      <c r="B58" t="s">
+        <v>160</v>
+      </c>
+      <c r="C58" t="s">
+        <v>11</v>
+      </c>
+      <c r="D58" s="1">
+        <v>46199</v>
+      </c>
+      <c r="E58" s="7">
+        <v>0</v>
+      </c>
+      <c r="F58">
+        <v>1</v>
+      </c>
+      <c r="G58">
+        <v>1</v>
+      </c>
+      <c r="H58">
+        <v>0</v>
+      </c>
+      <c r="I58">
+        <v>0</v>
+      </c>
+      <c r="J58">
+        <v>1</v>
+      </c>
+      <c r="K58">
+        <v>1</v>
+      </c>
+      <c r="P58" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q58">
+        <v>8</v>
+      </c>
+      <c r="R58">
+        <v>11</v>
+      </c>
+      <c r="S58">
+        <v>3</v>
+      </c>
+      <c r="T58">
+        <v>5</v>
+      </c>
+      <c r="U58">
+        <v>20</v>
+      </c>
+      <c r="V58">
+        <v>11</v>
+      </c>
+      <c r="W58">
+        <v>2</v>
+      </c>
+      <c r="X58">
+        <v>8</v>
+      </c>
+      <c r="Y58">
+        <v>1</v>
+      </c>
+      <c r="Z58">
+        <v>2</v>
+      </c>
+      <c r="AA58">
+        <v>0</v>
+      </c>
+      <c r="AB58">
+        <v>0</v>
+      </c>
+      <c r="AC58">
+        <v>1.21</v>
+      </c>
+      <c r="AD58">
+        <v>0.64</v>
+      </c>
+      <c r="AE58">
+        <v>2.4</v>
+      </c>
+      <c r="AF58">
+        <v>3.2</v>
+      </c>
+      <c r="AG58">
+        <v>3.1</v>
+      </c>
+      <c r="AH58">
+        <v>2.4</v>
+      </c>
+      <c r="AI58">
+        <v>3.5</v>
+      </c>
+      <c r="AJ58">
+        <v>3.3</v>
+      </c>
+      <c r="AK58">
+        <v>2.4</v>
+      </c>
+      <c r="AL58">
+        <v>3.6</v>
+      </c>
+      <c r="AM58">
+        <v>3.4</v>
+      </c>
+      <c r="AN58">
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="AO58">
+        <v>3.35</v>
+      </c>
+      <c r="AP58">
+        <v>3.13</v>
+      </c>
+    </row>
+    <row r="59" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>266</v>
+      </c>
+      <c r="B59" t="s">
+        <v>107</v>
+      </c>
+      <c r="C59" t="s">
+        <v>50</v>
+      </c>
+      <c r="D59" s="1">
+        <v>46199</v>
+      </c>
+      <c r="E59" s="7">
+        <v>0</v>
+      </c>
+      <c r="F59">
+        <v>1</v>
+      </c>
+      <c r="G59">
+        <v>3</v>
+      </c>
+      <c r="H59">
+        <v>0</v>
+      </c>
+      <c r="I59">
+        <v>2</v>
+      </c>
+      <c r="J59">
+        <v>1</v>
+      </c>
+      <c r="K59">
+        <v>1</v>
+      </c>
+      <c r="P59" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q59">
+        <v>10</v>
+      </c>
+      <c r="R59">
+        <v>20</v>
+      </c>
+      <c r="S59">
+        <v>4</v>
+      </c>
+      <c r="T59">
+        <v>7</v>
+      </c>
+      <c r="U59">
+        <v>11</v>
+      </c>
+      <c r="V59">
+        <v>10</v>
+      </c>
+      <c r="W59">
+        <v>4</v>
+      </c>
+      <c r="X59">
+        <v>6</v>
+      </c>
+      <c r="Y59">
+        <v>0</v>
+      </c>
+      <c r="Z59">
+        <v>0</v>
+      </c>
+      <c r="AA59">
+        <v>0</v>
+      </c>
+      <c r="AB59">
+        <v>0</v>
+      </c>
+      <c r="AC59">
+        <v>0.62</v>
+      </c>
+      <c r="AD59">
+        <v>1.84</v>
+      </c>
+      <c r="AE59">
+        <v>21</v>
+      </c>
+      <c r="AF59">
+        <v>8</v>
+      </c>
+      <c r="AG59">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="AH59">
+        <v>25</v>
+      </c>
+      <c r="AI59">
+        <v>11</v>
+      </c>
+      <c r="AJ59">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="AK59">
+        <v>21</v>
+      </c>
+      <c r="AL59">
+        <v>12</v>
+      </c>
+      <c r="AM59">
+        <v>1.17</v>
+      </c>
+      <c r="AN59">
+        <v>16.63</v>
+      </c>
+      <c r="AO59">
+        <v>8.56</v>
+      </c>
+      <c r="AP59">
+        <v>1.1399999999999999</v>
+      </c>
+    </row>
+    <row r="60" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>266</v>
+      </c>
+      <c r="B60" t="s">
+        <v>134</v>
+      </c>
+      <c r="C60" t="s">
+        <v>149</v>
+      </c>
+      <c r="D60" s="1">
+        <v>46199</v>
+      </c>
+      <c r="E60" s="7">
+        <v>0.125</v>
+      </c>
+      <c r="F60">
+        <v>0</v>
+      </c>
+      <c r="G60">
+        <v>0</v>
+      </c>
+      <c r="H60">
+        <v>0</v>
+      </c>
+      <c r="I60">
+        <v>0</v>
+      </c>
+      <c r="J60">
+        <v>0</v>
+      </c>
+      <c r="K60">
+        <v>0</v>
+      </c>
+      <c r="P60" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q60">
+        <v>7</v>
+      </c>
+      <c r="R60">
+        <v>12</v>
+      </c>
+      <c r="S60">
+        <v>2</v>
+      </c>
+      <c r="T60">
+        <v>5</v>
+      </c>
+      <c r="U60">
+        <v>9</v>
+      </c>
+      <c r="V60">
+        <v>6</v>
+      </c>
+      <c r="W60">
+        <v>1</v>
+      </c>
+      <c r="X60">
+        <v>3</v>
+      </c>
+      <c r="Y60">
+        <v>1</v>
+      </c>
+      <c r="Z60">
+        <v>1</v>
+      </c>
+      <c r="AA60">
+        <v>0</v>
+      </c>
+      <c r="AB60">
+        <v>0</v>
+      </c>
+      <c r="AC60">
+        <v>0.24</v>
+      </c>
+      <c r="AD60">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AE60">
+        <v>2.5499999999999998</v>
+      </c>
+      <c r="AF60">
+        <v>2.4</v>
+      </c>
+      <c r="AG60">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AH60">
+        <v>2.64</v>
+      </c>
+      <c r="AI60">
+        <v>2.5</v>
+      </c>
+      <c r="AJ60">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="AK60">
+        <v>2.63</v>
+      </c>
+      <c r="AL60">
+        <v>2.4500000000000002</v>
+      </c>
+      <c r="AM60">
+        <v>4.33</v>
+      </c>
+      <c r="AN60">
+        <v>2.52</v>
+      </c>
+      <c r="AO60">
+        <v>2.34</v>
+      </c>
+      <c r="AP60">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="61" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>266</v>
+      </c>
+      <c r="B61" t="s">
+        <v>10</v>
+      </c>
+      <c r="C61" t="s">
+        <v>257</v>
+      </c>
+      <c r="D61" s="1">
+        <v>46199</v>
+      </c>
+      <c r="E61" s="7">
+        <v>0.125</v>
+      </c>
+      <c r="F61">
+        <v>3</v>
+      </c>
+      <c r="G61">
+        <v>2</v>
+      </c>
+      <c r="H61">
+        <v>2</v>
+      </c>
+      <c r="I61">
+        <v>1</v>
+      </c>
+      <c r="J61">
+        <v>1</v>
+      </c>
+      <c r="K61">
+        <v>1</v>
+      </c>
+      <c r="P61" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q61">
+        <v>9</v>
+      </c>
+      <c r="R61">
+        <v>18</v>
+      </c>
+      <c r="S61">
+        <v>3</v>
+      </c>
+      <c r="T61">
+        <v>7</v>
+      </c>
+      <c r="U61">
+        <v>13</v>
+      </c>
+      <c r="V61">
+        <v>13</v>
+      </c>
+      <c r="W61">
+        <v>2</v>
+      </c>
+      <c r="X61">
+        <v>9</v>
+      </c>
+      <c r="Y61">
+        <v>0</v>
+      </c>
+      <c r="Z61">
+        <v>1</v>
+      </c>
+      <c r="AA61">
+        <v>0</v>
+      </c>
+      <c r="AB61">
+        <v>0</v>
+      </c>
+      <c r="AC61">
+        <v>3</v>
+      </c>
+      <c r="AD61">
+        <v>2.12</v>
+      </c>
+      <c r="AE61">
+        <v>3.2</v>
+      </c>
+      <c r="AF61">
+        <v>4</v>
+      </c>
+      <c r="AG61">
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="AH61">
+        <v>3.25</v>
+      </c>
+      <c r="AI61">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AJ61">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="AK61">
+        <v>3.6</v>
+      </c>
+      <c r="AL61">
+        <v>4</v>
+      </c>
+      <c r="AM61">
+        <v>2.1</v>
+      </c>
+      <c r="AN61">
+        <v>3.22</v>
+      </c>
+      <c r="AO61">
+        <v>3.81</v>
+      </c>
+      <c r="AP61">
+        <v>2.04</v>
+      </c>
+    </row>
+    <row r="62" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>266</v>
+      </c>
+      <c r="B62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C62" t="s">
+        <v>60</v>
+      </c>
+      <c r="D62" s="1">
+        <v>46199</v>
+      </c>
+      <c r="E62" s="7">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F62">
+        <v>1</v>
+      </c>
+      <c r="G62">
+        <v>4</v>
+      </c>
+      <c r="H62">
+        <v>1</v>
+      </c>
+      <c r="I62">
+        <v>3</v>
+      </c>
+      <c r="J62">
+        <v>0</v>
+      </c>
+      <c r="K62">
+        <v>1</v>
+      </c>
+      <c r="P62" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q62">
+        <v>10</v>
+      </c>
+      <c r="R62">
+        <v>18</v>
+      </c>
+      <c r="S62">
+        <v>4</v>
+      </c>
+      <c r="T62">
+        <v>9</v>
+      </c>
+      <c r="U62">
+        <v>9</v>
+      </c>
+      <c r="V62">
+        <v>11</v>
+      </c>
+      <c r="W62">
+        <v>4</v>
+      </c>
+      <c r="X62">
+        <v>5</v>
+      </c>
+      <c r="Y62">
+        <v>1</v>
+      </c>
+      <c r="Z62">
+        <v>1</v>
+      </c>
+      <c r="AA62">
+        <v>0</v>
+      </c>
+      <c r="AB62">
+        <v>0</v>
+      </c>
+      <c r="AC62">
+        <v>1.7</v>
+      </c>
+      <c r="AD62">
+        <v>1.5</v>
+      </c>
+      <c r="AE62">
+        <v>7</v>
+      </c>
+      <c r="AF62">
+        <v>5.5</v>
+      </c>
+      <c r="AG62">
+        <v>1.36</v>
+      </c>
+      <c r="AH62">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="AI62">
+        <v>6</v>
+      </c>
+      <c r="AJ62">
+        <v>1.39</v>
+      </c>
+      <c r="AK62">
+        <v>8</v>
+      </c>
+      <c r="AL62">
+        <v>6</v>
+      </c>
+      <c r="AM62">
+        <v>1.4</v>
+      </c>
+      <c r="AN62">
+        <v>7.02</v>
+      </c>
+      <c r="AO62">
+        <v>5.44</v>
+      </c>
+      <c r="AP62">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="63" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>266</v>
+      </c>
+      <c r="B63" t="s">
+        <v>81</v>
+      </c>
+      <c r="C63" t="s">
+        <v>1</v>
+      </c>
+      <c r="D63" s="1">
+        <v>46199</v>
+      </c>
+      <c r="E63" s="7">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F63">
+        <v>5</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63">
+        <v>1</v>
+      </c>
+      <c r="I63">
+        <v>0</v>
+      </c>
+      <c r="J63">
+        <v>4</v>
+      </c>
+      <c r="K63">
+        <v>0</v>
+      </c>
+      <c r="P63" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q63">
+        <v>28</v>
+      </c>
+      <c r="R63">
+        <v>6</v>
+      </c>
+      <c r="S63">
+        <v>12</v>
+      </c>
+      <c r="T63">
+        <v>1</v>
+      </c>
+      <c r="U63">
+        <v>10</v>
+      </c>
+      <c r="V63">
+        <v>11</v>
+      </c>
+      <c r="W63">
+        <v>12</v>
+      </c>
+      <c r="X63">
+        <v>3</v>
+      </c>
+      <c r="Y63">
+        <v>2</v>
+      </c>
+      <c r="Z63">
+        <v>2</v>
+      </c>
+      <c r="AA63">
+        <v>0</v>
+      </c>
+      <c r="AB63">
+        <v>1</v>
+      </c>
+      <c r="AC63">
+        <v>3.01</v>
+      </c>
+      <c r="AD63">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="AE63">
+        <v>1.2</v>
+      </c>
+      <c r="AF63">
+        <v>7</v>
+      </c>
+      <c r="AG63">
+        <v>12</v>
+      </c>
+      <c r="AH63">
+        <v>1.23</v>
+      </c>
+      <c r="AI63">
+        <v>8</v>
+      </c>
+      <c r="AJ63">
+        <v>14.5</v>
+      </c>
+      <c r="AK63">
+        <v>1.23</v>
+      </c>
+      <c r="AL63">
+        <v>7.5</v>
+      </c>
+      <c r="AM63">
+        <v>15</v>
+      </c>
+      <c r="AN63">
+        <v>1.2</v>
+      </c>
+      <c r="AO63">
+        <v>6.88</v>
+      </c>
+      <c r="AP63">
+        <v>13.06</v>
+      </c>
+    </row>
+    <row r="64" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>266</v>
+      </c>
+      <c r="B64" t="s">
+        <v>97</v>
+      </c>
+      <c r="C64" t="s">
+        <v>83</v>
+      </c>
+      <c r="D64" s="1">
+        <v>46200</v>
+      </c>
+      <c r="E64" s="7">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F64">
+        <v>0</v>
+      </c>
+      <c r="G64">
+        <v>0</v>
+      </c>
+      <c r="H64">
+        <v>0</v>
+      </c>
+      <c r="I64">
+        <v>0</v>
+      </c>
+      <c r="J64">
+        <v>0</v>
+      </c>
+      <c r="K64">
+        <v>0</v>
+      </c>
+      <c r="P64" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q64">
+        <v>15</v>
+      </c>
+      <c r="R64">
+        <v>7</v>
+      </c>
+      <c r="S64">
+        <v>2</v>
+      </c>
+      <c r="T64">
+        <v>3</v>
+      </c>
+      <c r="U64">
+        <v>10</v>
+      </c>
+      <c r="V64">
+        <v>16</v>
+      </c>
+      <c r="W64">
+        <v>4</v>
+      </c>
+      <c r="X64">
+        <v>2</v>
+      </c>
+      <c r="Y64">
+        <v>1</v>
+      </c>
+      <c r="Z64">
+        <v>3</v>
+      </c>
+      <c r="AA64">
+        <v>0</v>
+      </c>
+      <c r="AB64">
+        <v>0</v>
+      </c>
+      <c r="AC64">
+        <v>1.39</v>
+      </c>
+      <c r="AD64">
+        <v>0.39</v>
+      </c>
+      <c r="AE64">
+        <v>2.5</v>
+      </c>
+      <c r="AF64">
+        <v>3.3</v>
+      </c>
+      <c r="AG64">
+        <v>2.88</v>
+      </c>
+      <c r="AH64">
+        <v>2.7</v>
+      </c>
+      <c r="AI64">
+        <v>3.6</v>
+      </c>
+      <c r="AJ64">
+        <v>2.8</v>
+      </c>
+      <c r="AK64">
+        <v>2.74</v>
+      </c>
+      <c r="AL64">
+        <v>3.5</v>
+      </c>
+      <c r="AM64">
+        <v>2.88</v>
+      </c>
+      <c r="AN64">
+        <v>2.5499999999999998</v>
+      </c>
+      <c r="AO64">
+        <v>3.29</v>
+      </c>
+      <c r="AP64">
+        <v>2.72</v>
+      </c>
+    </row>
+    <row r="65" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>266</v>
+      </c>
+      <c r="B65" t="s">
+        <v>130</v>
+      </c>
+      <c r="C65" t="s">
+        <v>44</v>
+      </c>
+      <c r="D65" s="1">
+        <v>46200</v>
+      </c>
+      <c r="E65" s="7">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F65">
+        <v>0</v>
+      </c>
+      <c r="G65">
+        <v>1</v>
+      </c>
+      <c r="H65">
+        <v>0</v>
+      </c>
+      <c r="I65">
+        <v>1</v>
+      </c>
+      <c r="J65">
+        <v>0</v>
+      </c>
+      <c r="K65">
+        <v>0</v>
+      </c>
+      <c r="P65" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q65">
+        <v>5</v>
+      </c>
+      <c r="R65">
+        <v>6</v>
+      </c>
+      <c r="S65">
+        <v>1</v>
+      </c>
+      <c r="T65">
+        <v>1</v>
+      </c>
+      <c r="U65">
+        <v>14</v>
+      </c>
+      <c r="V65">
+        <v>14</v>
+      </c>
+      <c r="W65">
+        <v>1</v>
+      </c>
+      <c r="X65">
+        <v>6</v>
+      </c>
+      <c r="Y65">
+        <v>3</v>
+      </c>
+      <c r="Z65">
+        <v>1</v>
+      </c>
+      <c r="AA65">
+        <v>1</v>
+      </c>
+      <c r="AB65">
+        <v>0</v>
+      </c>
+      <c r="AC65">
+        <v>0.2</v>
+      </c>
+      <c r="AD65">
+        <v>0.86</v>
+      </c>
+      <c r="AE65">
+        <v>6</v>
+      </c>
+      <c r="AF65">
+        <v>3.6</v>
+      </c>
+      <c r="AG65">
+        <v>1.65</v>
+      </c>
+      <c r="AH65">
+        <v>6.4</v>
+      </c>
+      <c r="AI65">
+        <v>3.75</v>
+      </c>
+      <c r="AJ65">
+        <v>1.71</v>
+      </c>
+      <c r="AK65">
+        <v>6.25</v>
+      </c>
+      <c r="AL65">
+        <v>3.75</v>
+      </c>
+      <c r="AM65">
+        <v>1.7</v>
+      </c>
+      <c r="AN65">
+        <v>5.65</v>
+      </c>
+      <c r="AO65">
+        <v>3.59</v>
+      </c>
+      <c r="AP65">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="66" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>266</v>
+      </c>
+      <c r="B66" t="s">
+        <v>117</v>
+      </c>
+      <c r="C66" t="s">
+        <v>152</v>
+      </c>
+      <c r="D66" s="1">
+        <v>46200</v>
+      </c>
+      <c r="E66" s="7">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="F66">
+        <v>1</v>
+      </c>
+      <c r="G66">
+        <v>1</v>
+      </c>
+      <c r="H66">
+        <v>1</v>
+      </c>
+      <c r="I66">
+        <v>1</v>
+      </c>
+      <c r="J66">
+        <v>0</v>
+      </c>
+      <c r="K66">
+        <v>0</v>
+      </c>
+      <c r="P66" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q66">
+        <v>15</v>
+      </c>
+      <c r="R66">
+        <v>13</v>
+      </c>
+      <c r="S66">
+        <v>3</v>
+      </c>
+      <c r="T66">
+        <v>4</v>
+      </c>
+      <c r="U66">
+        <v>11</v>
+      </c>
+      <c r="V66">
+        <v>16</v>
+      </c>
+      <c r="W66">
+        <v>8</v>
+      </c>
+      <c r="X66">
+        <v>2</v>
+      </c>
+      <c r="Y66">
+        <v>3</v>
+      </c>
+      <c r="Z66">
+        <v>4</v>
+      </c>
+      <c r="AA66">
+        <v>0</v>
+      </c>
+      <c r="AB66">
+        <v>0</v>
+      </c>
+      <c r="AC66">
+        <v>0.84</v>
+      </c>
+      <c r="AD66">
+        <v>1.97</v>
+      </c>
+      <c r="AE66">
+        <v>2.63</v>
+      </c>
+      <c r="AF66">
+        <v>2.63</v>
+      </c>
+      <c r="AG66">
+        <v>3.4</v>
+      </c>
+      <c r="AH66">
+        <v>2.68</v>
+      </c>
+      <c r="AI66">
+        <v>2.82</v>
+      </c>
+      <c r="AJ66">
+        <v>3.65</v>
+      </c>
+      <c r="AK66">
+        <v>2.7</v>
+      </c>
+      <c r="AL66">
+        <v>2.8</v>
+      </c>
+      <c r="AM66">
+        <v>3.66</v>
+      </c>
+      <c r="AN66">
+        <v>2.58</v>
+      </c>
+      <c r="AO66">
+        <v>2.64</v>
+      </c>
+      <c r="AP66">
+        <v>3.38</v>
+      </c>
+    </row>
+    <row r="67" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>266</v>
+      </c>
+      <c r="B67" t="s">
+        <v>167</v>
+      </c>
+      <c r="C67" t="s">
+        <v>36</v>
+      </c>
+      <c r="D67" s="1">
+        <v>46200</v>
+      </c>
+      <c r="E67" s="7">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="F67">
+        <v>1</v>
+      </c>
+      <c r="G67">
+        <v>5</v>
+      </c>
+      <c r="H67">
+        <v>0</v>
+      </c>
+      <c r="I67">
+        <v>1</v>
+      </c>
+      <c r="J67">
+        <v>1</v>
+      </c>
+      <c r="K67">
+        <v>4</v>
+      </c>
+      <c r="P67" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q67">
+        <v>6</v>
+      </c>
+      <c r="R67">
+        <v>35</v>
+      </c>
+      <c r="S67">
+        <v>2</v>
+      </c>
+      <c r="T67">
+        <v>10</v>
+      </c>
+      <c r="U67">
+        <v>10</v>
+      </c>
+      <c r="V67">
+        <v>7</v>
+      </c>
+      <c r="W67">
+        <v>5</v>
+      </c>
+      <c r="X67">
+        <v>8</v>
+      </c>
+      <c r="Y67">
+        <v>2</v>
+      </c>
+      <c r="Z67">
+        <v>0</v>
+      </c>
+      <c r="AA67">
+        <v>0</v>
+      </c>
+      <c r="AB67">
+        <v>0</v>
+      </c>
+      <c r="AC67">
+        <v>0.24</v>
+      </c>
+      <c r="AD67">
+        <v>3.64</v>
+      </c>
+      <c r="AE67">
+        <v>13</v>
+      </c>
+      <c r="AF67">
+        <v>8.5</v>
+      </c>
+      <c r="AG67">
+        <v>1.17</v>
+      </c>
+      <c r="AH67">
+        <v>15.5</v>
+      </c>
+      <c r="AI67">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="AJ67">
+        <v>1.2</v>
+      </c>
+      <c r="AK67">
+        <v>15</v>
+      </c>
+      <c r="AL67">
+        <v>9</v>
+      </c>
+      <c r="AM67">
+        <v>1.19</v>
+      </c>
+      <c r="AN67">
+        <v>13.28</v>
+      </c>
+      <c r="AO67">
+        <v>8.14</v>
+      </c>
+      <c r="AP67">
+        <v>1.17</v>
+      </c>
+    </row>
+    <row r="68" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>266</v>
+      </c>
+      <c r="B68" t="s">
+        <v>47</v>
+      </c>
+      <c r="C68" t="s">
+        <v>113</v>
+      </c>
+      <c r="D68" s="1">
+        <v>46200</v>
+      </c>
+      <c r="E68" s="7">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="F68">
+        <v>2</v>
+      </c>
+      <c r="G68">
+        <v>1</v>
+      </c>
+      <c r="H68">
+        <v>1</v>
+      </c>
+      <c r="I68">
+        <v>0</v>
+      </c>
+      <c r="J68">
+        <v>1</v>
+      </c>
+      <c r="K68">
+        <v>1</v>
+      </c>
+      <c r="P68" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q68">
+        <v>8</v>
+      </c>
+      <c r="R68">
+        <v>6</v>
+      </c>
+      <c r="S68">
+        <v>4</v>
+      </c>
+      <c r="T68">
+        <v>1</v>
+      </c>
+      <c r="U68">
+        <v>9</v>
+      </c>
+      <c r="V68">
+        <v>13</v>
+      </c>
+      <c r="W68">
+        <v>3</v>
+      </c>
+      <c r="X68">
+        <v>2</v>
+      </c>
+      <c r="Y68">
+        <v>1</v>
+      </c>
+      <c r="Z68">
+        <v>1</v>
+      </c>
+      <c r="AA68">
+        <v>0</v>
+      </c>
+      <c r="AB68">
+        <v>0</v>
+      </c>
+      <c r="AC68">
+        <v>0.42</v>
+      </c>
+      <c r="AD68">
+        <v>0.64</v>
+      </c>
+      <c r="AE68">
+        <v>1.8</v>
+      </c>
+      <c r="AF68">
+        <v>3.1</v>
+      </c>
+      <c r="AG68">
+        <v>5.75</v>
+      </c>
+      <c r="AH68">
+        <v>1.84</v>
+      </c>
+      <c r="AI68">
+        <v>3.3</v>
+      </c>
+      <c r="AJ68">
+        <v>6.2</v>
+      </c>
+      <c r="AK68">
+        <v>1.87</v>
+      </c>
+      <c r="AL68">
+        <v>3.35</v>
+      </c>
+      <c r="AM68">
+        <v>5.75</v>
+      </c>
+      <c r="AN68">
+        <v>1.79</v>
+      </c>
+      <c r="AO68">
+        <v>3.16</v>
+      </c>
+      <c r="AP68">
+        <v>5.39</v>
+      </c>
+    </row>
+    <row r="69" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>266</v>
+      </c>
+      <c r="B69" t="s">
+        <v>28</v>
+      </c>
+      <c r="C69" t="s">
+        <v>58</v>
+      </c>
+      <c r="D69" s="1">
+        <v>46200</v>
+      </c>
+      <c r="E69" s="7">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="F69">
+        <v>0</v>
+      </c>
+      <c r="G69">
+        <v>2</v>
+      </c>
+      <c r="H69">
+        <v>0</v>
+      </c>
+      <c r="I69">
+        <v>0</v>
+      </c>
+      <c r="J69">
+        <v>0</v>
+      </c>
+      <c r="K69">
+        <v>2</v>
+      </c>
+      <c r="P69" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q69">
+        <v>13</v>
+      </c>
+      <c r="R69">
+        <v>17</v>
+      </c>
+      <c r="S69">
+        <v>2</v>
+      </c>
+      <c r="T69">
+        <v>6</v>
+      </c>
+      <c r="U69">
+        <v>16</v>
+      </c>
+      <c r="V69">
+        <v>13</v>
+      </c>
+      <c r="W69">
+        <v>3</v>
+      </c>
+      <c r="X69">
+        <v>7</v>
+      </c>
+      <c r="Y69">
+        <v>2</v>
+      </c>
+      <c r="Z69">
+        <v>1</v>
+      </c>
+      <c r="AA69">
+        <v>0</v>
+      </c>
+      <c r="AB69">
+        <v>0</v>
+      </c>
+      <c r="AC69">
+        <v>0.66</v>
+      </c>
+      <c r="AD69">
+        <v>1.57</v>
+      </c>
+      <c r="AE69">
+        <v>17</v>
+      </c>
+      <c r="AF69">
+        <v>8.5</v>
+      </c>
+      <c r="AG69">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="AH69">
+        <v>23</v>
+      </c>
+      <c r="AI69">
+        <v>9.4</v>
+      </c>
+      <c r="AJ69">
+        <v>1.17</v>
+      </c>
+      <c r="AK69">
+        <v>20</v>
+      </c>
+      <c r="AL69">
+        <v>9.5</v>
+      </c>
+      <c r="AM69">
+        <v>1.17</v>
+      </c>
+      <c r="AN69">
+        <v>16.53</v>
+      </c>
+      <c r="AO69">
+        <v>8.4499999999999993</v>
+      </c>
+      <c r="AP69">
+        <v>1.1399999999999999</v>
+      </c>
+    </row>
+    <row r="70" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>266</v>
+      </c>
+      <c r="B70" t="s">
+        <v>132</v>
+      </c>
+      <c r="C70" t="s">
+        <v>64</v>
+      </c>
+      <c r="D70" s="1">
+        <v>46201</v>
+      </c>
+      <c r="E70" s="7">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="F70">
+        <v>0</v>
+      </c>
+      <c r="G70">
+        <v>0</v>
+      </c>
+      <c r="H70">
+        <v>0</v>
+      </c>
+      <c r="I70">
+        <v>0</v>
+      </c>
+      <c r="J70">
+        <v>0</v>
+      </c>
+      <c r="K70">
+        <v>0</v>
+      </c>
+      <c r="P70" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q70">
+        <v>24</v>
+      </c>
+      <c r="R70">
+        <v>13</v>
+      </c>
+      <c r="S70">
+        <v>6</v>
+      </c>
+      <c r="T70">
+        <v>2</v>
+      </c>
+      <c r="U70">
+        <v>12</v>
+      </c>
+      <c r="V70">
+        <v>6</v>
+      </c>
+      <c r="W70">
+        <v>5</v>
+      </c>
+      <c r="X70">
+        <v>2</v>
+      </c>
+      <c r="Y70">
+        <v>1</v>
+      </c>
+      <c r="Z70">
+        <v>0</v>
+      </c>
+      <c r="AA70">
+        <v>0</v>
+      </c>
+      <c r="AB70">
+        <v>0</v>
+      </c>
+      <c r="AC70">
+        <v>1.7</v>
+      </c>
+      <c r="AD70">
+        <v>0.92</v>
+      </c>
+      <c r="AE70">
+        <v>4</v>
+      </c>
+      <c r="AF70">
+        <v>4</v>
+      </c>
+      <c r="AG70">
+        <v>1.8</v>
+      </c>
+      <c r="AH70">
+        <v>4.3</v>
+      </c>
+      <c r="AI70">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AJ70">
+        <v>1.89</v>
+      </c>
+      <c r="AK70">
+        <v>4</v>
+      </c>
+      <c r="AL70">
+        <v>4</v>
+      </c>
+      <c r="AM70">
+        <v>1.9</v>
+      </c>
+      <c r="AN70">
+        <v>3.83</v>
+      </c>
+      <c r="AO70">
+        <v>3.84</v>
+      </c>
+      <c r="AP70">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="71" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>266</v>
+      </c>
+      <c r="B71" t="s">
+        <v>3</v>
+      </c>
+      <c r="C71" t="s">
+        <v>155</v>
+      </c>
+      <c r="D71" s="1">
+        <v>46201</v>
+      </c>
+      <c r="E71" s="7">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="F71">
+        <v>3</v>
+      </c>
+      <c r="G71">
+        <v>1</v>
+      </c>
+      <c r="H71">
+        <v>0</v>
+      </c>
+      <c r="I71">
+        <v>1</v>
+      </c>
+      <c r="J71">
+        <v>3</v>
+      </c>
+      <c r="K71">
+        <v>0</v>
+      </c>
+      <c r="P71" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q71">
+        <v>19</v>
+      </c>
+      <c r="R71">
+        <v>3</v>
+      </c>
+      <c r="S71">
+        <v>4</v>
+      </c>
+      <c r="T71">
+        <v>1</v>
+      </c>
+      <c r="U71">
+        <v>6</v>
+      </c>
+      <c r="V71">
+        <v>16</v>
+      </c>
+      <c r="W71">
+        <v>2</v>
+      </c>
+      <c r="X71">
+        <v>4</v>
+      </c>
+      <c r="Y71">
+        <v>3</v>
+      </c>
+      <c r="Z71">
+        <v>2</v>
+      </c>
+      <c r="AA71">
+        <v>0</v>
+      </c>
+      <c r="AB71">
+        <v>0</v>
+      </c>
+      <c r="AC71">
+        <v>2.17</v>
+      </c>
+      <c r="AD71">
+        <v>0.2</v>
+      </c>
+      <c r="AE71">
+        <v>1.67</v>
+      </c>
+      <c r="AF71">
+        <v>3.8</v>
+      </c>
+      <c r="AG71">
+        <v>5.25</v>
+      </c>
+      <c r="AH71">
+        <v>1.71</v>
+      </c>
+      <c r="AI71">
+        <v>4</v>
+      </c>
+      <c r="AJ71">
+        <v>5.7</v>
+      </c>
+      <c r="AK71">
+        <v>1.68</v>
+      </c>
+      <c r="AL71">
+        <v>4</v>
+      </c>
+      <c r="AM71">
+        <v>5.5</v>
+      </c>
+      <c r="AN71">
+        <v>1.64</v>
+      </c>
+      <c r="AO71">
+        <v>3.79</v>
+      </c>
+      <c r="AP71">
+        <v>5.23</v>
+      </c>
+    </row>
+    <row r="72" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>266</v>
+      </c>
+      <c r="B72" t="s">
+        <v>87</v>
+      </c>
+      <c r="C72" t="s">
+        <v>33</v>
+      </c>
+      <c r="D72" s="1">
+        <v>46201</v>
+      </c>
+      <c r="E72" s="7">
+        <v>0.125</v>
+      </c>
+      <c r="F72">
+        <v>3</v>
+      </c>
+      <c r="G72">
+        <v>3</v>
+      </c>
+      <c r="H72">
+        <v>1</v>
+      </c>
+      <c r="I72">
+        <v>1</v>
+      </c>
+      <c r="J72">
+        <v>2</v>
+      </c>
+      <c r="K72">
+        <v>2</v>
+      </c>
+      <c r="P72" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q72">
+        <v>12</v>
+      </c>
+      <c r="R72">
+        <v>10</v>
+      </c>
+      <c r="S72">
+        <v>5</v>
+      </c>
+      <c r="T72">
+        <v>3</v>
+      </c>
+      <c r="U72">
+        <v>3</v>
+      </c>
+      <c r="V72">
+        <v>7</v>
+      </c>
+      <c r="W72">
+        <v>0</v>
+      </c>
+      <c r="X72">
+        <v>3</v>
+      </c>
+      <c r="Y72">
+        <v>0</v>
+      </c>
+      <c r="Z72">
+        <v>1</v>
+      </c>
+      <c r="AA72">
+        <v>0</v>
+      </c>
+      <c r="AB72">
+        <v>0</v>
+      </c>
+      <c r="AC72">
+        <v>1.67</v>
+      </c>
+      <c r="AD72">
+        <v>1.49</v>
+      </c>
+      <c r="AE72">
+        <v>3.5</v>
+      </c>
+      <c r="AF72">
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="AG72">
+        <v>3.6</v>
+      </c>
+      <c r="AH72">
+        <v>3.7</v>
+      </c>
+      <c r="AI72">
+        <v>2.14</v>
+      </c>
+      <c r="AJ72">
+        <v>3.75</v>
+      </c>
+      <c r="AK72">
+        <v>3.55</v>
+      </c>
+      <c r="AL72">
+        <v>2.15</v>
+      </c>
+      <c r="AM72">
+        <v>3.75</v>
+      </c>
+      <c r="AN72">
+        <v>3.33</v>
+      </c>
+      <c r="AO72">
+        <v>2.09</v>
+      </c>
+      <c r="AP72">
+        <v>3.45</v>
+      </c>
+    </row>
+    <row r="73" spans="1:42" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>266</v>
+      </c>
+      <c r="B73" t="s">
+        <v>150</v>
+      </c>
+      <c r="C73" t="s">
+        <v>136</v>
+      </c>
+      <c r="D73" s="1">
+        <v>46201</v>
+      </c>
+      <c r="E73" s="7">
+        <v>0.125</v>
+      </c>
+      <c r="F73">
+        <v>1</v>
+      </c>
+      <c r="G73">
+        <v>3</v>
+      </c>
+      <c r="H73">
+        <v>0</v>
+      </c>
+      <c r="I73">
+        <v>2</v>
+      </c>
+      <c r="J73">
+        <v>1</v>
+      </c>
+      <c r="K73">
+        <v>1</v>
+      </c>
+      <c r="P73" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q73">
+        <v>5</v>
+      </c>
+      <c r="R73">
+        <v>12</v>
+      </c>
+      <c r="S73">
+        <v>1</v>
+      </c>
+      <c r="T73">
+        <v>4</v>
+      </c>
+      <c r="U73">
+        <v>13</v>
+      </c>
+      <c r="V73">
+        <v>7</v>
+      </c>
+      <c r="W73">
+        <v>2</v>
+      </c>
+      <c r="X73">
+        <v>6</v>
+      </c>
+      <c r="Y73">
+        <v>3</v>
+      </c>
+      <c r="Z73">
+        <v>0</v>
+      </c>
+      <c r="AA73">
+        <v>0</v>
+      </c>
+      <c r="AB73">
+        <v>0</v>
+      </c>
+      <c r="AC73">
+        <v>0.76</v>
+      </c>
+      <c r="AD73">
+        <v>2.13</v>
+      </c>
+      <c r="AE73">
+        <v>21</v>
+      </c>
+      <c r="AF73">
+        <v>9</v>
+      </c>
+      <c r="AG73">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="AH73">
+        <v>25</v>
+      </c>
+      <c r="AI73">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="AJ73">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="AK73">
+        <v>21</v>
+      </c>
+      <c r="AL73">
+        <v>9</v>
+      </c>
+      <c r="AM73">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="AN73">
+        <v>19.03</v>
+      </c>
+      <c r="AO73">
+        <v>8.4499999999999993</v>
+      </c>
+      <c r="AP73">
+        <v>1.1299999999999999</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AP49">
-    <sortCondition ref="D2:D49"/>
-    <sortCondition ref="E2:E49"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AP73">
+    <sortCondition ref="D2:D73"/>
+    <sortCondition ref="E2:E73"/>
   </sortState>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>